<commit_message>
App 2.8.1: klasseoppgavene i appen er versjon 6, rettede nedtrekkslister i Excel
</commit_message>
<xml_diff>
--- a/pensum/ma01/MA01_Hva_er_markedsforing_Oppgaver_v6.xlsx
+++ b/pensum/ma01/MA01_Hva_er_markedsforing_Oppgaver_v6.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="145">
   <si>
     <t xml:space="preserve">Hva er markedsføring? Oppgaver til kapittel 1</t>
   </si>
@@ -65,18 +65,33 @@
     <t xml:space="preserve">Dette er øvingsmateriell til repetisjons- og øvingsstøtte. I besvarelser, caser, prosjektoppgaver og eksamen gjelder lærebøkene og oppgitte primærkilder.</t>
   </si>
   <si>
+    <t xml:space="preserve">Bedriftsmarkedet</t>
+  </si>
+  <si>
     <t xml:space="preserve">Oppgave 1A: Ida har åtte forespørsler: hvem kjøper, og i hvilket marked?</t>
   </si>
   <si>
+    <t xml:space="preserve">Mellomhandlermarkedet</t>
+  </si>
+  <si>
     <t xml:space="preserve">Alene, i par eller i gruppe, slik du vil.</t>
   </si>
   <si>
+    <t xml:space="preserve">Det offentlige markedet</t>
+  </si>
+  <si>
     <t xml:space="preserve">Situasjonen</t>
   </si>
   <si>
+    <t xml:space="preserve">Organisasjonsmarkedet</t>
+  </si>
+  <si>
     <t xml:space="preserve">Det er mandag morgen hos Nordlys Elektro. Ida (kalkulatør) har åtte forespørsler på bordet og tid til å regne på to av dem denne uka. Kari (daglig leder) sier på morgenmøtet: «Vi trenger ikke markedsføring, vi har nok å gjøre.» Plasser hver forespørsel i riktig hovedmarked, finn hvilken betydning av «marked» som brukes, regn markedet for husstandene i kroner, og svar Kari.</t>
   </si>
   <si>
+    <t xml:space="preserve">Forbrukermarkedet</t>
+  </si>
+  <si>
     <t xml:space="preserve">Begrepene du trenger</t>
   </si>
   <si>
@@ -156,6 +171,15 @@
   </si>
   <si>
     <t xml:space="preserve">Gule celler fyller du inn. Grønne regnes ut av arket. Sjekken til høyre forteller om svaret stemmer, og hva du bør se på hvis ikke.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kjøperne (betydning 1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Omsetningen i et år (betydning 2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tilbudet akkurat nå (betydning 3)</t>
   </si>
   <si>
     <t xml:space="preserve">Oppgave 1B: Nordlys' markeder: hvor avhengig er Kari av byggherrene?</t>
@@ -245,12 +269,27 @@
     <t xml:space="preserve">d) Kari sier: «Vi lever av byggherrene.» Bruk tallene fra b og c: stemmer det, hva er risikoen, og hvilket hovedmarked ville du vokse i? To–tre setninger.</t>
   </si>
   <si>
+    <t xml:space="preserve">Produksjonsorientering</t>
+  </si>
+  <si>
     <t xml:space="preserve">Oppgave 1C: Mandagsmøtet hos Nordlys: fem forslag, og et slagord</t>
   </si>
   <si>
+    <t xml:space="preserve">Produktorientering</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Salgsorientering</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Markedsorientering</t>
+  </si>
+  <si>
     <t xml:space="preserve">I fjor leverte Ida tre anbud på ladeanlegg til borettslag og vant ingen av dem, selv om Nordlys' anlegg ble vurdert som teknisk best alle tre gangene. Det er 22 borettslag i nedslagsfeltet. På mandagsmøtet kommer fem forslag til hva Nordlys skal gjøre. Samtidig har Kari skrevet et løfte på nettsiden, Kystfiber vil samarbeide, og Fjell Elektro vurderer et slagord. Sett navn på grunnholdningene og kravene, og skriv spørsmålene Ida bør stille styret.</t>
   </si>
   <si>
+    <t xml:space="preserve">Helhetlig markedsorientering</t>
+  </si>
+  <si>
     <t xml:space="preserve">Salgsorientering finner kjøpere til bedriftens produkter; markedsorientering finner de rette produktene til kjøperne. Helhetlig markedsorientering stiller tre krav samtidig: ekstern og intern markedsføring henger sammen, langsiktige relasjoner (relasjonsmarkedsføring, som gir synergi), og markedsføring innenfor lov, etikk og miljøhensyn. Kjøpers marked: stor konkurranse, bedriften lytter til kunden. Selgers marked: liten konkurranse, bedriften styrer. Lovgivningen er som regel bare en minimumsløsning.</t>
   </si>
   <si>
@@ -296,10 +335,34 @@
     <t xml:space="preserve">Mai hos Nordlys: alle vil ha ladepunkt før ferien, og Nordlys setter leveringstiden</t>
   </si>
   <si>
+    <t xml:space="preserve">Ekstern og intern markedsføring henger sammen</t>
+  </si>
+  <si>
     <t xml:space="preserve">Kari: «Vi følger loven, så vi kan kalle oss bærekraftige.» Hva sier boka?</t>
   </si>
   <si>
+    <t xml:space="preserve">Relasjonsmarkedsføring</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lov, etikk og miljø</t>
+  </si>
+  <si>
     <t xml:space="preserve">Skriv tre ting Ida bør spørre et borettslagsstyre om før hun skriver neste tilbud, og si hvilket av forslagene 1–5 du bygger på.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kjøpers marked</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Selgers marked</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Riktig: loven bestemmer hva som er bærekraftig</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Loven er som regel bare en minimumsløsning; over den skal bedriften også tenke på det allmenne vel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bærekraft gjelder bare store selskaper</t>
   </si>
   <si>
     <t xml:space="preserve">Fasit, kapittel 1</t>
@@ -585,7 +648,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -608,6 +671,10 @@
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -1054,7 +1121,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="B2:G41"/>
+  <dimension ref="B1:Z49"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
@@ -1062,345 +1129,523 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="56"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="26" min="26" style="0" width="13"/>
   </cols>
   <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="Z1" s="0" t="s">
+        <v>13</v>
+      </c>
+    </row>
     <row r="2" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C2" s="5"/>
       <c r="D2" s="5"/>
       <c r="E2" s="5"/>
       <c r="F2" s="5"/>
       <c r="G2" s="5"/>
+      <c r="Z2" s="6" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B3" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="C3" s="6"/>
-      <c r="D3" s="6"/>
-      <c r="E3" s="6"/>
-      <c r="F3" s="6"/>
-      <c r="G3" s="6"/>
+      <c r="B3" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" s="7"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="7"/>
+      <c r="G3" s="7"/>
+      <c r="Z3" s="6" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" s="8"/>
+      <c r="D4" s="8"/>
+      <c r="E4" s="8"/>
+      <c r="F4" s="8"/>
+      <c r="G4" s="8"/>
+      <c r="Z4" s="6" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B5" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
+      <c r="Z5" s="6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B6" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" s="8"/>
+      <c r="D6" s="8"/>
+      <c r="E6" s="8"/>
+      <c r="F6" s="8"/>
+      <c r="G6" s="8"/>
+      <c r="Z6" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B7" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" s="9"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9"/>
+      <c r="G7" s="9"/>
+      <c r="Z7" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="7"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
-    </row>
-    <row r="5" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B5" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="C5" s="8"/>
-      <c r="D5" s="8"/>
-      <c r="E5" s="8"/>
-      <c r="F5" s="8"/>
-      <c r="G5" s="8"/>
-    </row>
-    <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B6" s="7" t="s">
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="Z8" s="0" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="7"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
-      <c r="G6" s="7"/>
-    </row>
-    <row r="7" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B7" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="C7" s="8"/>
-      <c r="D7" s="8"/>
-      <c r="E7" s="8"/>
-      <c r="F7" s="8"/>
-      <c r="G7" s="8"/>
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="C9" s="8"/>
+      <c r="D9" s="8"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="8"/>
+      <c r="G9" s="8"/>
+      <c r="Z9" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="7"/>
     </row>
     <row r="10" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B10" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="C10" s="8"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="8"/>
-      <c r="F10" s="8"/>
-      <c r="G10" s="8"/>
+      <c r="B10" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="C10" s="9"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="9"/>
+      <c r="G10" s="9"/>
+      <c r="Z10" s="6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="Z11" s="0" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B12" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="C12" s="9"/>
-      <c r="D12" s="9"/>
-      <c r="E12" s="9"/>
-      <c r="F12" s="9"/>
-      <c r="G12" s="9"/>
+      <c r="B12" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="C12" s="10"/>
+      <c r="D12" s="10"/>
+      <c r="E12" s="10"/>
+      <c r="F12" s="10"/>
+      <c r="G12" s="10"/>
+      <c r="Z12" s="6" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B13" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="C13" s="11"/>
-      <c r="G13" s="12" t="str">
+      <c r="B13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="C13" s="12"/>
+      <c r="G13" s="13" t="str">
         <f aca="false">IF(C13="","Velg i nedtrekksmenyen.",IF(C13="Forbrukermarkedet","Riktig. En husholdning som kjøper til eget konsum, amatør i kjøpet (1.4.5).","Ikke riktig. En husholdning som kjøper til eget konsum, amatør i kjøpet (1.4.5)."))</f>
         <v>Velg i nedtrekksmenyen.</v>
       </c>
+      <c r="Z13" s="6" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B14" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="C14" s="11"/>
-      <c r="G14" s="12" t="str">
+      <c r="B14" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="C14" s="12"/>
+      <c r="G14" s="13" t="str">
         <f aca="false">IF(C14="","Velg i nedtrekksmenyen.",IF(C14="Bedriftsmarkedet","Riktig. Kjøper i næring, som del av egen leveranse (1.4.1).","Ikke riktig. Kjøper i næring, som del av egen leveranse (1.4.1)."))</f>
         <v>Velg i nedtrekksmenyen.</v>
       </c>
+      <c r="Z14" s="6" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B15" s="10" t="s">
-        <v>24</v>
-      </c>
-      <c r="C15" s="11"/>
-      <c r="G15" s="12" t="str">
+      <c r="B15" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="C15" s="12"/>
+      <c r="G15" s="13" t="str">
         <f aca="false">IF(C15="","Velg i nedtrekksmenyen.",IF(C15="Det offentlige markedet","Riktig. Kommunal forvaltning. Boka plasserer forvaltningen i stat, fylke og kommune her (1.4.3).","Ikke riktig. Kommunal forvaltning. Boka plasserer forvaltningen i stat, fylke og kommune her (1.4.3)."))</f>
         <v>Velg i nedtrekksmenyen.</v>
       </c>
+      <c r="Z15" s="6" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B16" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="C16" s="11"/>
-      <c r="G16" s="12" t="str">
+      <c r="B16" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C16" s="12"/>
+      <c r="G16" s="13" t="str">
         <f aca="false">IF(C16="","Velg i nedtrekksmenyen.",IF(C16="Organisasjonsmarkedet","Riktig. En frivillig organisasjon (1.4.4).","Ikke riktig. En frivillig organisasjon (1.4.4)."))</f>
         <v>Velg i nedtrekksmenyen.</v>
       </c>
+      <c r="Z16" s="6" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B17" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="C17" s="11"/>
-      <c r="G17" s="12" t="str">
+      <c r="B17" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="C17" s="12"/>
+      <c r="G17" s="13" t="str">
         <f aca="false">IF(C17="","Velg i nedtrekksmenyen.",IF(C17="Mellomhandlermarkedet","Riktig. Detaljisten er ikke sluttbruker; den kjøper for å selge videre (1.4.2). At sluttkunden er en huseier, gjør ikke byggvarehuset til forbruker.","Ikke riktig. Detaljisten er ikke sluttbruker; den kjøper for å selge videre (1.4.2). At sluttkunden er en huseier, gjør ikke byggvarehuset til forbruker."))</f>
         <v>Velg i nedtrekksmenyen.</v>
       </c>
+      <c r="Z17" s="6" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B18" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="C18" s="11"/>
-      <c r="G18" s="12" t="str">
+      <c r="B18" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="C18" s="12"/>
+      <c r="G18" s="13" t="str">
         <f aca="false">IF(C18="","Velg i nedtrekksmenyen.",IF(C18="Bedriftsmarkedet","Riktig. Offentlig næringsdrift hører til bedriftsmarkedet (1.4.1). Det offentlige markedet er forvaltningen, ikke selskapene det offentlige eier (1.4.3).","Ikke riktig. Offentlig næringsdrift hører til bedriftsmarkedet (1.4.1). Det offentlige markedet er forvaltningen, ikke selskapene det offentlige eier (1.4.3)."))</f>
         <v>Velg i nedtrekksmenyen.</v>
       </c>
+      <c r="Z18" s="6" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B19" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="C19" s="11"/>
-      <c r="G19" s="12" t="str">
+      <c r="B19" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="C19" s="12"/>
+      <c r="G19" s="13" t="str">
         <f aca="false">IF(C19="","Velg i nedtrekksmenyen.",IF(C19="Bedriftsmarkedet","Riktig. Byggherren kjøper i næring; bygget skal leies ut (1.4.1).","Ikke riktig. Byggherren kjøper i næring; bygget skal leies ut (1.4.1)."))</f>
         <v>Velg i nedtrekksmenyen.</v>
       </c>
+      <c r="Z19" s="6" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B20" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="C20" s="11"/>
-      <c r="G20" s="12" t="str">
+      <c r="B20" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="C20" s="12"/>
+      <c r="G20" s="13" t="str">
         <f aca="false">IF(C20="","Velg i nedtrekksmenyen.",IF(C20="Det offentlige markedet","Riktig. Statlig forvaltning: departementer, direktorater og etater (1.4.3).","Ikke riktig. Statlig forvaltning: departementer, direktorater og etater (1.4.3)."))</f>
         <v>Velg i nedtrekksmenyen.</v>
       </c>
+      <c r="Z20" s="6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="Z21" s="0" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B22" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="C22" s="7"/>
-      <c r="D22" s="7"/>
-      <c r="E22" s="7"/>
-      <c r="F22" s="7"/>
-      <c r="G22" s="7"/>
+      <c r="B22" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="C22" s="8"/>
+      <c r="D22" s="8"/>
+      <c r="E22" s="8"/>
+      <c r="F22" s="8"/>
+      <c r="G22" s="8"/>
+      <c r="Z22" s="6" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B23" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="C23" s="8"/>
-      <c r="D23" s="8"/>
-      <c r="E23" s="8"/>
-      <c r="F23" s="8"/>
-      <c r="G23" s="8"/>
+      <c r="B23" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C23" s="9"/>
+      <c r="D23" s="9"/>
+      <c r="E23" s="9"/>
+      <c r="F23" s="9"/>
+      <c r="G23" s="9"/>
+      <c r="Z23" s="6" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B24" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="C24" s="11"/>
-      <c r="G24" s="12" t="str">
+      <c r="B24" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="C24" s="12"/>
+      <c r="G24" s="13" t="str">
         <f aca="false">IF(C24="","Velg i nedtrekksmenyen.",IF(C24="Kjøperne (betydning 1)","Riktig. Antall kjøpere, både de som kjøper og de som kan komme til å kjøpe (1.1, betydning 1).","Ikke riktig. Antall kjøpere, både de som kjøper og de som kan komme til å kjøpe (1.1, betydning 1)."))</f>
         <v>Velg i nedtrekksmenyen.</v>
       </c>
+      <c r="Z24" s="6" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B25" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="C25" s="11"/>
-      <c r="G25" s="12" t="str">
+      <c r="B25" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="C25" s="12"/>
+      <c r="G25" s="13" t="str">
         <f aca="false">IF(C25="","Velg i nedtrekksmenyen.",IF(C25="Omsetningen i et år (betydning 2)","Riktig. Kroner per år er den samlede omsetningen i løpet av et år (1.1, betydning 2).","Ikke riktig. Kroner per år er den samlede omsetningen i løpet av et år (1.1, betydning 2)."))</f>
         <v>Velg i nedtrekksmenyen.</v>
       </c>
+      <c r="Z25" s="6" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B26" s="10" t="s">
-        <v>34</v>
-      </c>
-      <c r="C26" s="11"/>
-      <c r="G26" s="12" t="str">
+      <c r="B26" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="C26" s="12"/>
+      <c r="G26" s="13" t="str">
         <f aca="false">IF(C26="","Velg i nedtrekksmenyen.",IF(C26="Tilbudet akkurat nå (betydning 3)","Riktig. Det samlede tilbudet på et bestemt tidspunkt (1.1, betydning 3).","Ikke riktig. Det samlede tilbudet på et bestemt tidspunkt (1.1, betydning 3)."))</f>
         <v>Velg i nedtrekksmenyen.</v>
       </c>
+      <c r="Z26" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="Z27" s="0" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B28" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="C28" s="7"/>
-      <c r="D28" s="7"/>
-      <c r="E28" s="7"/>
-      <c r="F28" s="7"/>
-      <c r="G28" s="7"/>
+      <c r="B28" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="C28" s="8"/>
+      <c r="D28" s="8"/>
+      <c r="E28" s="8"/>
+      <c r="F28" s="8"/>
+      <c r="G28" s="8"/>
+      <c r="Z28" s="6" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B29" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="C29" s="8"/>
-      <c r="D29" s="8"/>
-      <c r="E29" s="8"/>
-      <c r="F29" s="8"/>
-      <c r="G29" s="8"/>
+      <c r="B29" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="C29" s="9"/>
+      <c r="D29" s="9"/>
+      <c r="E29" s="9"/>
+      <c r="F29" s="9"/>
+      <c r="G29" s="9"/>
+      <c r="Z29" s="6" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B30" s="10" t="s">
-        <v>37</v>
-      </c>
-      <c r="C30" s="13"/>
-      <c r="D30" s="14" t="s">
-        <v>38</v>
-      </c>
-      <c r="G30" s="12" t="str">
+      <c r="B30" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="C30" s="14"/>
+      <c r="D30" s="15" t="s">
+        <v>43</v>
+      </c>
+      <c r="G30" s="13" t="str">
         <f aca="false">IF(C30="","Skriv svaret i den gule cellen.",IF(C30=(ROUND(9200*0.08,0)),"Riktig.",IF(ABS(C30-(ROUND(9200*0.8,0)))&lt;=0,"Du har brukt 80 %. Det er 8 %, altså 0,08.",IF(ABS(C30-(9200))&lt;=0,"Det er alle husstandene (betydning 1). Bare 8 % kjøper i året.","Ikke riktig ennå. Se på regnestykket øverst på fanen, og sjekk at du har med alle leddene."))))</f>
         <v>Skriv svaret i den gule cellen.</v>
       </c>
+      <c r="Z30" s="6" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B31" s="10" t="s">
-        <v>39</v>
-      </c>
-      <c r="C31" s="13"/>
-      <c r="D31" s="14" t="s">
-        <v>40</v>
-      </c>
-      <c r="G31" s="12" t="str">
+      <c r="B31" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="C31" s="14"/>
+      <c r="D31" s="15" t="s">
+        <v>45</v>
+      </c>
+      <c r="G31" s="13" t="str">
         <f aca="false">IF(C31="","Skriv svaret i den gule cellen.",IF(C31=(ROUND(9200*0.08*14000,0)),"Riktig.",IF(ABS(C31-(9200*14000))&lt;=0,"Du har ganget alle 9 200 med 14 000. Bare 736 kjøper i året.",IF(ABS(C31-(ROUND(9200*0.08,0)))&lt;=0,"Det er antall husstander som kjøper. Gang med snittjobben, 14 000 kr.","Ikke riktig ennå. Se på regnestykket øverst på fanen, og sjekk at du har med alle leddene."))))</f>
         <v>Skriv svaret i den gule cellen.</v>
       </c>
+      <c r="Z31" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="Z32" s="0" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B33" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="C33" s="8"/>
-      <c r="D33" s="8"/>
-      <c r="E33" s="8"/>
-      <c r="F33" s="8"/>
-      <c r="G33" s="8"/>
+      <c r="B33" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="C33" s="9"/>
+      <c r="D33" s="9"/>
+      <c r="E33" s="9"/>
+      <c r="F33" s="9"/>
+      <c r="G33" s="9"/>
+      <c r="Z33" s="6" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B34" s="15"/>
-      <c r="C34" s="15"/>
-      <c r="D34" s="15"/>
-      <c r="E34" s="15"/>
-      <c r="F34" s="15"/>
-      <c r="G34" s="15"/>
+      <c r="B34" s="16"/>
+      <c r="C34" s="16"/>
+      <c r="D34" s="16"/>
+      <c r="E34" s="16"/>
+      <c r="F34" s="16"/>
+      <c r="G34" s="16"/>
+      <c r="Z34" s="6" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="35" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B35" s="15"/>
-      <c r="C35" s="15"/>
-      <c r="D35" s="15"/>
-      <c r="E35" s="15"/>
-      <c r="F35" s="15"/>
-      <c r="G35" s="15"/>
+      <c r="B35" s="16"/>
+      <c r="C35" s="16"/>
+      <c r="D35" s="16"/>
+      <c r="E35" s="16"/>
+      <c r="F35" s="16"/>
+      <c r="G35" s="16"/>
+      <c r="Z35" s="6" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B36" s="15"/>
-      <c r="C36" s="15"/>
-      <c r="D36" s="15"/>
-      <c r="E36" s="15"/>
-      <c r="F36" s="15"/>
-      <c r="G36" s="15"/>
+      <c r="B36" s="16"/>
+      <c r="C36" s="16"/>
+      <c r="D36" s="16"/>
+      <c r="E36" s="16"/>
+      <c r="F36" s="16"/>
+      <c r="G36" s="16"/>
+      <c r="Z36" s="6" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="37" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B37" s="16" t="str">
+      <c r="B37" s="17" t="str">
         <f aca="false">IF(LEN(B34)&lt;40,"",IF(AND(ISNUMBER(SEARCH("behov",B34)),ISNUMBER(SEARCH("lønnsom",B34))),"Bra: du bruker definisjonen med behov og lønnsomhet. Sjekk at eksemplet ditt viser at Nordlys velger kunder når Ida velger hva hun regner på.",IF(OR(ISNUMBER(SEARCH("behov",B34)),ISNUMBER(SEARCH("lønnsom",B34))),"Du er på sporet. Definisjonen har to deler: avdekke og imøtekomme ønsker og behov, og gjøre det på en lønnsom måte. Ta med begge, og et eksempel fra forespørslene.","Tips: markedsføring er alle aktivitetene for å avdekke og imøtekomme markedets ønsker og behov på en lønnsom måte. Når Ida velger to av åtte forespørsler, velger Nordlys kunder. Det er markedsføring uten annonse.")))</f>
         <v/>
       </c>
-      <c r="C37" s="16"/>
-      <c r="D37" s="16"/>
-      <c r="E37" s="16"/>
-      <c r="F37" s="16"/>
-      <c r="G37" s="16"/>
+      <c r="C37" s="17"/>
+      <c r="D37" s="17"/>
+      <c r="E37" s="17"/>
+      <c r="F37" s="17"/>
+      <c r="G37" s="17"/>
+      <c r="Z37" s="6" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B38" s="17" t="s">
-        <v>42</v>
-      </c>
-      <c r="C38" s="11"/>
+      <c r="B38" s="18" t="s">
+        <v>47</v>
+      </c>
+      <c r="C38" s="12"/>
+      <c r="Z38" s="6" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="39" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B39" s="18" t="str">
+      <c r="B39" s="19" t="str">
         <f aca="false">IF(C38="JA","Hint: Spør for hver forespørsel: kjøper de til eget bruk, i næring, for å selge videre, som forvaltning eller som organisasjon? Fjellkraft Nett AS driver næring selv om kommunen eier det. Byggvarehuset kjøper for å selge videre. Markedet i kroner: 9 200 × 0,08 = 736 husstander, × 14 000 kr = 10 304 000 kr.","")</f>
         <v/>
       </c>
-      <c r="C39" s="18"/>
-      <c r="D39" s="18"/>
-      <c r="E39" s="18"/>
-      <c r="F39" s="18"/>
-      <c r="G39" s="18"/>
+      <c r="C39" s="19"/>
+      <c r="D39" s="19"/>
+      <c r="E39" s="19"/>
+      <c r="F39" s="19"/>
+      <c r="G39" s="19"/>
+      <c r="Z39" s="6" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="Z40" s="0" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="41" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B41" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="C41" s="6"/>
-      <c r="D41" s="6"/>
-      <c r="E41" s="6"/>
-      <c r="F41" s="6"/>
-      <c r="G41" s="6"/>
+      <c r="B41" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="C41" s="7"/>
+      <c r="D41" s="7"/>
+      <c r="E41" s="7"/>
+      <c r="F41" s="7"/>
+      <c r="G41" s="7"/>
+      <c r="Z41" s="6" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="Z42" s="0" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="Z43" s="0" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="Z44" s="0" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="Z45" s="0" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="Z46" s="0" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="Z47" s="0" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="Z48" s="0" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="Z49" s="0" t="s">
+        <v>51</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="18">
@@ -1529,47 +1774,47 @@
   </conditionalFormatting>
   <dataValidations count="12">
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C13" type="list">
-      <formula1>"Bedriftsmarkedet,Mellomhandlermarkedet,Det offentlige markedet,Organisasjonsmarkedet,Forbrukermarkedet"</formula1>
+      <formula1>$Z$1:$Z$5</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C14" type="list">
-      <formula1>"Bedriftsmarkedet,Mellomhandlermarkedet,Det offentlige markedet,Organisasjonsmarkedet,Forbrukermarkedet"</formula1>
+      <formula1>$Z$6:$Z$10</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C15" type="list">
-      <formula1>"Bedriftsmarkedet,Mellomhandlermarkedet,Det offentlige markedet,Organisasjonsmarkedet,Forbrukermarkedet"</formula1>
+      <formula1>$Z$11:$Z$15</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C16" type="list">
-      <formula1>"Bedriftsmarkedet,Mellomhandlermarkedet,Det offentlige markedet,Organisasjonsmarkedet,Forbrukermarkedet"</formula1>
+      <formula1>$Z$16:$Z$20</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C17" type="list">
-      <formula1>"Bedriftsmarkedet,Mellomhandlermarkedet,Det offentlige markedet,Organisasjonsmarkedet,Forbrukermarkedet"</formula1>
+      <formula1>$Z$21:$Z$25</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C18" type="list">
-      <formula1>"Bedriftsmarkedet,Mellomhandlermarkedet,Det offentlige markedet,Organisasjonsmarkedet,Forbrukermarkedet"</formula1>
+      <formula1>$Z$26:$Z$30</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C19" type="list">
-      <formula1>"Bedriftsmarkedet,Mellomhandlermarkedet,Det offentlige markedet,Organisasjonsmarkedet,Forbrukermarkedet"</formula1>
+      <formula1>$Z$31:$Z$35</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C20" type="list">
-      <formula1>"Bedriftsmarkedet,Mellomhandlermarkedet,Det offentlige markedet,Organisasjonsmarkedet,Forbrukermarkedet"</formula1>
+      <formula1>$Z$36:$Z$40</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C24" type="list">
-      <formula1>"Kjøperne (betydning 1),Omsetningen i et år (betydning 2),Tilbudet akkurat nå (betydning 3)"</formula1>
+      <formula1>$Z$41:$Z$43</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C25" type="list">
-      <formula1>"Kjøperne (betydning 1),Omsetningen i et år (betydning 2),Tilbudet akkurat nå (betydning 3)"</formula1>
+      <formula1>$Z$44:$Z$46</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C26" type="list">
-      <formula1>"Kjøperne (betydning 1),Omsetningen i et år (betydning 2),Tilbudet akkurat nå (betydning 3)"</formula1>
+      <formula1>$Z$47:$Z$49</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C38" type="list">
@@ -1592,7 +1837,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="B2:G43"/>
+  <dimension ref="B1:Z43"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
@@ -1600,353 +1845,454 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="56"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="26" min="26" style="0" width="13"/>
   </cols>
   <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="Z1" s="0" t="s">
+        <v>13</v>
+      </c>
+    </row>
     <row r="2" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="5" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="C2" s="5"/>
       <c r="D2" s="5"/>
       <c r="E2" s="5"/>
       <c r="F2" s="5"/>
       <c r="G2" s="5"/>
+      <c r="Z2" s="6" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B3" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="C3" s="6"/>
-      <c r="D3" s="6"/>
-      <c r="E3" s="6"/>
-      <c r="F3" s="6"/>
-      <c r="G3" s="6"/>
+      <c r="B3" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" s="7"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="7"/>
+      <c r="G3" s="7"/>
+      <c r="Z3" s="6" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" s="8"/>
+      <c r="D4" s="8"/>
+      <c r="E4" s="8"/>
+      <c r="F4" s="8"/>
+      <c r="G4" s="8"/>
+      <c r="Z4" s="6" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B5" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
+      <c r="Z5" s="6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B6" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" s="8"/>
+      <c r="D6" s="8"/>
+      <c r="E6" s="8"/>
+      <c r="F6" s="8"/>
+      <c r="G6" s="8"/>
+      <c r="Z6" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B7" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="C7" s="9"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9"/>
+      <c r="G7" s="9"/>
+      <c r="Z7" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="7"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
-    </row>
-    <row r="5" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B5" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="C5" s="8"/>
-      <c r="D5" s="8"/>
-      <c r="E5" s="8"/>
-      <c r="F5" s="8"/>
-      <c r="G5" s="8"/>
-    </row>
-    <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B6" s="7" t="s">
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="Z8" s="0" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="7"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
-      <c r="G6" s="7"/>
-    </row>
-    <row r="7" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B7" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="C7" s="8"/>
-      <c r="D7" s="8"/>
-      <c r="E7" s="8"/>
-      <c r="F7" s="8"/>
-      <c r="G7" s="8"/>
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B9" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="7"/>
+      <c r="B9" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="C9" s="8"/>
+      <c r="D9" s="8"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="8"/>
+      <c r="G9" s="8"/>
+      <c r="Z9" s="6" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B10" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="C10" s="8"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="8"/>
-      <c r="F10" s="8"/>
-      <c r="G10" s="8"/>
+      <c r="B10" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="C10" s="9"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="9"/>
+      <c r="G10" s="9"/>
+      <c r="Z10" s="6" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="19" t="s">
-        <v>49</v>
-      </c>
-      <c r="C11" s="20" t="s">
-        <v>50</v>
+      <c r="B11" s="20" t="s">
+        <v>57</v>
+      </c>
+      <c r="C11" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="Z11" s="6" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="21" t="s">
-        <v>51</v>
-      </c>
-      <c r="C12" s="22" t="n">
+      <c r="B12" s="22" t="s">
+        <v>59</v>
+      </c>
+      <c r="C12" s="23" t="n">
         <v>10500000</v>
       </c>
+      <c r="Z12" s="6" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="21" t="s">
-        <v>52</v>
-      </c>
-      <c r="C13" s="22" t="n">
+      <c r="B13" s="22" t="s">
+        <v>60</v>
+      </c>
+      <c r="C13" s="23" t="n">
         <v>4400000</v>
       </c>
+      <c r="Z13" s="6" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="21" t="s">
-        <v>53</v>
-      </c>
-      <c r="C14" s="22" t="n">
+      <c r="B14" s="22" t="s">
+        <v>61</v>
+      </c>
+      <c r="C14" s="23" t="n">
         <v>1650000</v>
       </c>
+      <c r="Z14" s="6" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="21" t="s">
-        <v>54</v>
-      </c>
-      <c r="C15" s="22" t="n">
+      <c r="B15" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="C15" s="23" t="n">
         <v>3800000</v>
       </c>
+      <c r="Z15" s="6" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="21" t="s">
-        <v>55</v>
-      </c>
-      <c r="C16" s="22" t="n">
+      <c r="B16" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C16" s="23" t="n">
         <v>1450000</v>
       </c>
+      <c r="Z16" s="6" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="21" t="s">
-        <v>56</v>
-      </c>
-      <c r="C17" s="22" t="n">
+      <c r="B17" s="22" t="s">
+        <v>64</v>
+      </c>
+      <c r="C17" s="23" t="n">
         <v>600000</v>
       </c>
+      <c r="Z17" s="6" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="21" t="s">
-        <v>57</v>
-      </c>
-      <c r="C18" s="23" t="n">
+      <c r="B18" s="22" t="s">
+        <v>65</v>
+      </c>
+      <c r="C18" s="24" t="n">
         <f aca="false">SUM(C12:C17)</f>
         <v>22400000</v>
       </c>
+      <c r="Z18" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="Z19" s="0" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B20" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="C20" s="7"/>
-      <c r="D20" s="7"/>
-      <c r="E20" s="7"/>
-      <c r="F20" s="7"/>
-      <c r="G20" s="7"/>
+      <c r="B20" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="C20" s="8"/>
+      <c r="D20" s="8"/>
+      <c r="E20" s="8"/>
+      <c r="F20" s="8"/>
+      <c r="G20" s="8"/>
+      <c r="Z20" s="6" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B21" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="C21" s="8"/>
-      <c r="D21" s="8"/>
-      <c r="E21" s="8"/>
-      <c r="F21" s="8"/>
-      <c r="G21" s="8"/>
+      <c r="B21" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="C21" s="9"/>
+      <c r="D21" s="9"/>
+      <c r="E21" s="9"/>
+      <c r="F21" s="9"/>
+      <c r="G21" s="9"/>
+      <c r="Z21" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="Z22" s="0" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B23" s="9" t="s">
-        <v>60</v>
-      </c>
-      <c r="C23" s="9"/>
-      <c r="D23" s="9"/>
-      <c r="E23" s="9"/>
-      <c r="F23" s="9"/>
-      <c r="G23" s="9"/>
+      <c r="B23" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="C23" s="10"/>
+      <c r="D23" s="10"/>
+      <c r="E23" s="10"/>
+      <c r="F23" s="10"/>
+      <c r="G23" s="10"/>
+      <c r="Z23" s="6" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B24" s="10" t="s">
-        <v>61</v>
-      </c>
-      <c r="C24" s="11"/>
-      <c r="G24" s="12" t="str">
+      <c r="B24" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="C24" s="12"/>
+      <c r="G24" s="13" t="str">
         <f aca="false">IF(C24="","Velg i nedtrekksmenyen.",IF(C24="Bedriftsmarkedet","Riktig. De kjøper i næring: bygget skal selges eller leies ut (1.4.1).","Ikke riktig. De kjøper i næring: bygget skal selges eller leies ut (1.4.1)."))</f>
         <v>Velg i nedtrekksmenyen.</v>
       </c>
+      <c r="Z24" s="6" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B25" s="10" t="s">
-        <v>62</v>
-      </c>
-      <c r="C25" s="11"/>
-      <c r="G25" s="12" t="str">
+      <c r="B25" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="C25" s="12"/>
+      <c r="G25" s="13" t="str">
         <f aca="false">IF(C25="","Velg i nedtrekksmenyen.",IF(C25="Bedriftsmarkedet","Riktig. Bedrifter som kjøper til egen drift, institusjonsvarer (1.4.1).","Ikke riktig. Bedrifter som kjøper til egen drift, institusjonsvarer (1.4.1)."))</f>
         <v>Velg i nedtrekksmenyen.</v>
       </c>
+      <c r="Z25" s="6" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B26" s="10" t="s">
-        <v>63</v>
-      </c>
-      <c r="C26" s="11"/>
-      <c r="G26" s="12" t="str">
+      <c r="B26" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="C26" s="12"/>
+      <c r="G26" s="13" t="str">
         <f aca="false">IF(C26="","Velg i nedtrekksmenyen.",IF(C26="Bedriftsmarkedet","Riktig. Offentlig næringsdrift er bedriftsmarkedet (1.4.1). Eieren avgjør ikke; virksomheten gjør det.","Ikke riktig. Offentlig næringsdrift er bedriftsmarkedet (1.4.1). Eieren avgjør ikke; virksomheten gjør det."))</f>
         <v>Velg i nedtrekksmenyen.</v>
       </c>
+      <c r="Z26" s="6" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B27" s="10" t="s">
-        <v>64</v>
-      </c>
-      <c r="C27" s="11"/>
-      <c r="G27" s="12" t="str">
+      <c r="B27" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="C27" s="12"/>
+      <c r="G27" s="13" t="str">
         <f aca="false">IF(C27="","Velg i nedtrekksmenyen.",IF(C27="Det offentlige markedet","Riktig. Forvaltningen på kommunalt og fylkeskommunalt nivå (1.4.3).","Ikke riktig. Forvaltningen på kommunalt og fylkeskommunalt nivå (1.4.3)."))</f>
         <v>Velg i nedtrekksmenyen.</v>
       </c>
+      <c r="Z27" s="6" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B28" s="10" t="s">
-        <v>65</v>
-      </c>
-      <c r="C28" s="11"/>
-      <c r="G28" s="12" t="str">
+      <c r="B28" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="C28" s="12"/>
+      <c r="G28" s="13" t="str">
         <f aca="false">IF(C28="","Velg i nedtrekksmenyen.",IF(C28="Forbrukermarkedet","Riktig. Enkeltpersoner og husholdninger som kjøper til eget konsum (1.4.5).","Ikke riktig. Enkeltpersoner og husholdninger som kjøper til eget konsum (1.4.5)."))</f>
         <v>Velg i nedtrekksmenyen.</v>
       </c>
+      <c r="Z28" s="6" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B29" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="C29" s="11"/>
-      <c r="G29" s="12" t="str">
+      <c r="B29" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="C29" s="12"/>
+      <c r="G29" s="13" t="str">
         <f aca="false">IF(C29="","Velg i nedtrekksmenyen.",IF(C29="Organisasjonsmarkedet","Riktig. Frivillige organisasjoner (1.4.4).","Ikke riktig. Frivillige organisasjoner (1.4.4)."))</f>
         <v>Velg i nedtrekksmenyen.</v>
       </c>
+      <c r="Z29" s="6" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="Z30" s="0" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B31" s="10" t="s">
-        <v>67</v>
-      </c>
-      <c r="C31" s="13"/>
-      <c r="D31" s="14" t="s">
-        <v>40</v>
-      </c>
-      <c r="G31" s="12" t="str">
+      <c r="B31" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="C31" s="14"/>
+      <c r="D31" s="15" t="s">
+        <v>45</v>
+      </c>
+      <c r="G31" s="13" t="str">
         <f aca="false">IF(C31="","Skriv svaret i den gule cellen.",IF(C31=(C12+C13+C14),"Riktig.",IF(ABS(C31-(C12+C13))&lt;=0,"Du har glemt Fjellkraft Nett AS. Nettselskapet er næringsdrift og hører til bedriftsmarkedet.",IF(ABS(C31-(C12+C13+C14+C15))&lt;=0,"Du har tatt med kommunen. Forvaltningen er det offentlige markedet, ikke bedriftsmarkedet.",IF(ABS(C31-(C12))&lt;=0,"Det er bare byggherrene. Bedriftsmarkedet har tre kundegrupper her.","Ikke riktig ennå. Se på regnestykket øverst på fanen, og sjekk at du har med alle leddene.")))))</f>
         <v>Skriv svaret i den gule cellen.</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B32" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="C32" s="24"/>
-      <c r="D32" s="14" t="s">
-        <v>69</v>
-      </c>
-      <c r="G32" s="12" t="str">
+      <c r="B32" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="C32" s="25"/>
+      <c r="D32" s="15" t="s">
+        <v>77</v>
+      </c>
+      <c r="G32" s="13" t="str">
         <f aca="false">IF(C32="","Skriv svaret i den gule cellen.",IF(C32=(ROUND((C12+C13+C14)/C18*100,0)),"Riktig.",IF(ABS(C32-(ROUND(C12/C18*100,0)))&lt;=0,"Det er byggherrenes andel alene. Her skal hele bedriftsmarkedet (a) deles på salgsinntekten.",IF(ABS(C32-(ROUND((C12+C13+C14+C15)/C18*100,0)))&lt;=0,"Du har tatt med kommunen i bedriftsmarkedet. Kommunen er det offentlige markedet.","Ikke riktig ennå. Se på regnestykket øverst på fanen, og sjekk at du har med alle leddene."))))</f>
         <v>Skriv svaret i den gule cellen.</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B33" s="10" t="s">
-        <v>70</v>
-      </c>
-      <c r="C33" s="24"/>
-      <c r="D33" s="14" t="s">
-        <v>69</v>
-      </c>
-      <c r="G33" s="12" t="str">
+      <c r="B33" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="C33" s="25"/>
+      <c r="D33" s="15" t="s">
+        <v>77</v>
+      </c>
+      <c r="G33" s="13" t="str">
         <f aca="false">IF(C33="","Skriv svaret i den gule cellen.",IF(C33=(ROUND(C12/C18*100,0)),"Riktig.",IF(ABS(C33-(ROUND(C12/(C12+C13+C14)*100,0)))&lt;=0,"Du har delt på bedriftsmarkedet, 16 550 000. Andelen skal regnes av hele salgsinntekten, 22 400 000.",IF(ABS(C33-(60))&lt;=0,"Det er bransjens tall, 59,6 %. Her spør vi om Nordlys: 10 500 000 delt på 22 400 000.","Ikke riktig ennå. Se på regnestykket øverst på fanen, og sjekk at du har med alle leddene."))))</f>
         <v>Skriv svaret i den gule cellen.</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B35" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="C35" s="8"/>
-      <c r="D35" s="8"/>
-      <c r="E35" s="8"/>
-      <c r="F35" s="8"/>
-      <c r="G35" s="8"/>
+      <c r="B35" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="C35" s="9"/>
+      <c r="D35" s="9"/>
+      <c r="E35" s="9"/>
+      <c r="F35" s="9"/>
+      <c r="G35" s="9"/>
     </row>
     <row r="36" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B36" s="15"/>
-      <c r="C36" s="15"/>
-      <c r="D36" s="15"/>
-      <c r="E36" s="15"/>
-      <c r="F36" s="15"/>
-      <c r="G36" s="15"/>
+      <c r="B36" s="16"/>
+      <c r="C36" s="16"/>
+      <c r="D36" s="16"/>
+      <c r="E36" s="16"/>
+      <c r="F36" s="16"/>
+      <c r="G36" s="16"/>
     </row>
     <row r="37" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B37" s="15"/>
-      <c r="C37" s="15"/>
-      <c r="D37" s="15"/>
-      <c r="E37" s="15"/>
-      <c r="F37" s="15"/>
-      <c r="G37" s="15"/>
+      <c r="B37" s="16"/>
+      <c r="C37" s="16"/>
+      <c r="D37" s="16"/>
+      <c r="E37" s="16"/>
+      <c r="F37" s="16"/>
+      <c r="G37" s="16"/>
     </row>
     <row r="38" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B38" s="15"/>
-      <c r="C38" s="15"/>
-      <c r="D38" s="15"/>
-      <c r="E38" s="15"/>
-      <c r="F38" s="15"/>
-      <c r="G38" s="15"/>
+      <c r="B38" s="16"/>
+      <c r="C38" s="16"/>
+      <c r="D38" s="16"/>
+      <c r="E38" s="16"/>
+      <c r="F38" s="16"/>
+      <c r="G38" s="16"/>
     </row>
     <row r="39" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B39" s="16" t="str">
+      <c r="B39" s="17" t="str">
         <f aca="false">IF(LEN(B36)&lt;40,"",IF(AND(ISNUMBER(SEARCH("byggherre",B36)),ISNUMBER(SEARCH("47",B36))),"Bra: du bruker 47 % og peker på byggherrene. Sjekk at du også sier hvilket marked du ville vokse i, og hvorfor det kjøper annerledes.",IF(OR(ISNUMBER(SEARCH("byggherre",B36)),ISNUMBER(SEARCH("47",B36))),"Du er på sporet. Bruk tallet: byggherrene er 47 % av salgsinntekten, mot 59,6 % i bransjen. Si hva som skjer når boligbyggingen stopper, og hvor du ville vokse.","Tips: 47 % av salgsinntekten kommer fra byggherrer og entreprenører, én kundegruppe som stopper når boligbyggingen stopper. Bransjen henter 59,6 % der, så Nordlys er litt mindre utsatt, men nesten halve omsetningen er i spill. Vekst kan ligge i service hos husstander og næringskunder, eller i anbud i det offentlige markedet.")))</f>
         <v/>
       </c>
-      <c r="C39" s="16"/>
-      <c r="D39" s="16"/>
-      <c r="E39" s="16"/>
-      <c r="F39" s="16"/>
-      <c r="G39" s="16"/>
+      <c r="C39" s="17"/>
+      <c r="D39" s="17"/>
+      <c r="E39" s="17"/>
+      <c r="F39" s="17"/>
+      <c r="G39" s="17"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B40" s="17" t="s">
-        <v>42</v>
-      </c>
-      <c r="C40" s="11"/>
+      <c r="B40" s="18" t="s">
+        <v>47</v>
+      </c>
+      <c r="C40" s="12"/>
     </row>
     <row r="41" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B41" s="18" t="str">
+      <c r="B41" s="19" t="str">
         <f aca="false">IF(C40="JA","Hint: Bedriftsmarkedet er byggherrer, næringskunder og Fjellkraft Nett: 10 500 000 + 4 400 000 + 1 650 000 = 16 550 000 kr. Delt på 22 400 000 er det 73,9 %, avrundet 74. Byggherrene alene: 10 500 000 / 22 400 000 = 46,9 %, avrundet 47.","")</f>
         <v/>
       </c>
-      <c r="C41" s="18"/>
-      <c r="D41" s="18"/>
-      <c r="E41" s="18"/>
-      <c r="F41" s="18"/>
-      <c r="G41" s="18"/>
+      <c r="C41" s="19"/>
+      <c r="D41" s="19"/>
+      <c r="E41" s="19"/>
+      <c r="F41" s="19"/>
+      <c r="G41" s="19"/>
     </row>
     <row r="43" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B43" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="C43" s="6"/>
-      <c r="D43" s="6"/>
-      <c r="E43" s="6"/>
-      <c r="F43" s="6"/>
-      <c r="G43" s="6"/>
+      <c r="B43" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="C43" s="7"/>
+      <c r="D43" s="7"/>
+      <c r="E43" s="7"/>
+      <c r="F43" s="7"/>
+      <c r="G43" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="16">
@@ -2041,27 +2387,27 @@
   </conditionalFormatting>
   <dataValidations count="7">
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C24" type="list">
-      <formula1>"Bedriftsmarkedet,Mellomhandlermarkedet,Det offentlige markedet,Organisasjonsmarkedet,Forbrukermarkedet"</formula1>
+      <formula1>$Z$1:$Z$5</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C25" type="list">
-      <formula1>"Bedriftsmarkedet,Mellomhandlermarkedet,Det offentlige markedet,Organisasjonsmarkedet,Forbrukermarkedet"</formula1>
+      <formula1>$Z$6:$Z$10</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C26" type="list">
-      <formula1>"Bedriftsmarkedet,Mellomhandlermarkedet,Det offentlige markedet,Organisasjonsmarkedet,Forbrukermarkedet"</formula1>
+      <formula1>$Z$11:$Z$15</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C27" type="list">
-      <formula1>"Bedriftsmarkedet,Mellomhandlermarkedet,Det offentlige markedet,Organisasjonsmarkedet,Forbrukermarkedet"</formula1>
+      <formula1>$Z$16:$Z$20</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C28" type="list">
-      <formula1>"Bedriftsmarkedet,Mellomhandlermarkedet,Det offentlige markedet,Organisasjonsmarkedet,Forbrukermarkedet"</formula1>
+      <formula1>$Z$21:$Z$25</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C29" type="list">
-      <formula1>"Bedriftsmarkedet,Mellomhandlermarkedet,Det offentlige markedet,Organisasjonsmarkedet,Forbrukermarkedet"</formula1>
+      <formula1>$Z$26:$Z$30</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C40" type="list">
@@ -2084,7 +2430,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="B2:G37"/>
+  <dimension ref="B1:Z41"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
@@ -2092,299 +2438,445 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="56"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="26" min="26" style="0" width="13"/>
   </cols>
   <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="Z1" s="0" t="s">
+        <v>80</v>
+      </c>
+    </row>
     <row r="2" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="5" t="s">
-        <v>72</v>
+        <v>81</v>
       </c>
       <c r="C2" s="5"/>
       <c r="D2" s="5"/>
       <c r="E2" s="5"/>
       <c r="F2" s="5"/>
       <c r="G2" s="5"/>
+      <c r="Z2" s="6" t="s">
+        <v>82</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B3" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="C3" s="6"/>
-      <c r="D3" s="6"/>
-      <c r="E3" s="6"/>
-      <c r="F3" s="6"/>
-      <c r="G3" s="6"/>
+      <c r="B3" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" s="7"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="7"/>
+      <c r="G3" s="7"/>
+      <c r="Z3" s="6" t="s">
+        <v>83</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B4" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4" s="7"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
+      <c r="B4" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" s="8"/>
+      <c r="D4" s="8"/>
+      <c r="E4" s="8"/>
+      <c r="F4" s="8"/>
+      <c r="G4" s="8"/>
+      <c r="Z4" s="6" t="s">
+        <v>84</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B5" s="8" t="s">
-        <v>73</v>
-      </c>
-      <c r="C5" s="8"/>
-      <c r="D5" s="8"/>
-      <c r="E5" s="8"/>
-      <c r="F5" s="8"/>
-      <c r="G5" s="8"/>
+      <c r="B5" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
+      <c r="Z5" s="6" t="s">
+        <v>86</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B6" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" s="7"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
-      <c r="G6" s="7"/>
+      <c r="B6" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" s="8"/>
+      <c r="D6" s="8"/>
+      <c r="E6" s="8"/>
+      <c r="F6" s="8"/>
+      <c r="G6" s="8"/>
+      <c r="Z6" s="6" t="s">
+        <v>80</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B7" s="8" t="s">
-        <v>74</v>
-      </c>
-      <c r="C7" s="8"/>
-      <c r="D7" s="8"/>
-      <c r="E7" s="8"/>
-      <c r="F7" s="8"/>
-      <c r="G7" s="8"/>
+      <c r="B7" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="C7" s="9"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9"/>
+      <c r="G7" s="9"/>
+      <c r="Z7" s="6" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="Z8" s="0" t="s">
+        <v>83</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B9" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="7"/>
+      <c r="B9" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="C9" s="8"/>
+      <c r="D9" s="8"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="8"/>
+      <c r="G9" s="8"/>
+      <c r="Z9" s="6" t="s">
+        <v>84</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B10" s="8" t="s">
-        <v>75</v>
-      </c>
-      <c r="C10" s="8"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="8"/>
-      <c r="F10" s="8"/>
-      <c r="G10" s="8"/>
+      <c r="B10" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="C10" s="9"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="9"/>
+      <c r="G10" s="9"/>
+      <c r="Z10" s="6" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="Z11" s="0" t="s">
+        <v>80</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B12" s="9" t="s">
-        <v>76</v>
-      </c>
-      <c r="C12" s="9"/>
-      <c r="D12" s="9"/>
-      <c r="E12" s="9"/>
-      <c r="F12" s="9"/>
-      <c r="G12" s="9"/>
+      <c r="B12" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="C12" s="10"/>
+      <c r="D12" s="10"/>
+      <c r="E12" s="10"/>
+      <c r="F12" s="10"/>
+      <c r="G12" s="10"/>
+      <c r="Z12" s="6" t="s">
+        <v>82</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B13" s="10" t="s">
-        <v>77</v>
-      </c>
-      <c r="C13" s="11"/>
-      <c r="G13" s="12" t="str">
+      <c r="B13" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="C13" s="12"/>
+      <c r="G13" s="13" t="str">
         <f aca="false">IF(C13="","Velg i nedtrekksmenyen.",IF(C13="Salgsorientering","Riktig. Starter med anlegget Nordlys har og leter etter flere kjøpere (1.2.3).","Ikke riktig. Starter med anlegget Nordlys har og leter etter flere kjøpere (1.2.3)."))</f>
         <v>Velg i nedtrekksmenyen.</v>
       </c>
+      <c r="Z13" s="6" t="s">
+        <v>83</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B14" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="C14" s="11"/>
-      <c r="G14" s="12" t="str">
+      <c r="B14" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="C14" s="12"/>
+      <c r="G14" s="13" t="str">
         <f aca="false">IF(C14="","Velg i nedtrekksmenyen.",IF(C14="Produktorientering","Riktig. Tar for gitt at markedet vil ha det beste produktet (1.2.2).","Ikke riktig. Tar for gitt at markedet vil ha det beste produktet (1.2.2)."))</f>
         <v>Velg i nedtrekksmenyen.</v>
       </c>
+      <c r="Z14" s="6" t="s">
+        <v>84</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B15" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="C15" s="11"/>
-      <c r="G15" s="12" t="str">
+      <c r="B15" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="C15" s="12"/>
+      <c r="G15" s="13" t="str">
         <f aca="false">IF(C15="","Velg i nedtrekksmenyen.",IF(C15="Produksjonsorientering","Riktig. Lave enhetskostnader og volum; billig og lett tilgjengelig (1.2.1).","Ikke riktig. Lave enhetskostnader og volum; billig og lett tilgjengelig (1.2.1)."))</f>
         <v>Velg i nedtrekksmenyen.</v>
       </c>
+      <c r="Z15" s="6" t="s">
+        <v>86</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B16" s="10" t="s">
-        <v>80</v>
-      </c>
-      <c r="C16" s="11"/>
-      <c r="G16" s="12" t="str">
+      <c r="B16" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="C16" s="12"/>
+      <c r="G16" s="13" t="str">
         <f aca="false">IF(C16="","Velg i nedtrekksmenyen.",IF(C16="Markedsorientering","Riktig. Finner de rette produktene til kjøperne; starter hos kunden (1.2.4).","Ikke riktig. Finner de rette produktene til kjøperne; starter hos kunden (1.2.4)."))</f>
         <v>Velg i nedtrekksmenyen.</v>
       </c>
+      <c r="Z16" s="6" t="s">
+        <v>80</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B17" s="10" t="s">
-        <v>81</v>
-      </c>
-      <c r="C17" s="11"/>
-      <c r="G17" s="12" t="str">
+      <c r="B17" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="C17" s="12"/>
+      <c r="G17" s="13" t="str">
         <f aca="false">IF(C17="","Velg i nedtrekksmenyen.",IF(C17="Helhetlig markedsorientering","Riktig. Det eksterne løftet må henge sammen med det de ansatte kjenner seg igjen i (1.2.5).","Ikke riktig. Det eksterne løftet må henge sammen med det de ansatte kjenner seg igjen i (1.2.5)."))</f>
         <v>Velg i nedtrekksmenyen.</v>
       </c>
+      <c r="Z17" s="6" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="Z18" s="0" t="s">
+        <v>83</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B19" s="9" t="s">
-        <v>82</v>
-      </c>
-      <c r="C19" s="9"/>
-      <c r="D19" s="9"/>
-      <c r="E19" s="9"/>
-      <c r="F19" s="9"/>
-      <c r="G19" s="9"/>
+      <c r="B19" s="10" t="s">
+        <v>95</v>
+      </c>
+      <c r="C19" s="10"/>
+      <c r="D19" s="10"/>
+      <c r="E19" s="10"/>
+      <c r="F19" s="10"/>
+      <c r="G19" s="10"/>
+      <c r="Z19" s="6" t="s">
+        <v>84</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B20" s="10" t="s">
-        <v>83</v>
-      </c>
-      <c r="C20" s="11"/>
-      <c r="G20" s="12" t="str">
+      <c r="B20" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="C20" s="12"/>
+      <c r="G20" s="13" t="str">
         <f aca="false">IF(C20="","Velg i nedtrekksmenyen.",IF(C20="Ekstern og intern markedsføring henger sammen","Riktig. De ansatte skal kjenne seg igjen i det bedriften lover kundene (1.2.5).","Ikke riktig. De ansatte skal kjenne seg igjen i det bedriften lover kundene (1.2.5)."))</f>
         <v>Velg i nedtrekksmenyen.</v>
       </c>
+      <c r="Z20" s="6" t="s">
+        <v>86</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B21" s="10" t="s">
-        <v>84</v>
-      </c>
-      <c r="C21" s="11"/>
-      <c r="G21" s="12" t="str">
+      <c r="B21" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="C21" s="12"/>
+      <c r="G21" s="13" t="str">
         <f aca="false">IF(C21="","Velg i nedtrekksmenyen.",IF(C21="Relasjonsmarkedsføring","Riktig. Langsiktig relasjon med en samarbeidspartner for å få mer ut av den samlede innsatsen; lykkes det, gir det synergi (1.2.5).","Ikke riktig. Langsiktig relasjon med en samarbeidspartner for å få mer ut av den samlede innsatsen; lykkes det, gir det synergi (1.2.5)."))</f>
         <v>Velg i nedtrekksmenyen.</v>
       </c>
+      <c r="Z21" s="6" t="s">
+        <v>80</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B22" s="10" t="s">
-        <v>85</v>
-      </c>
-      <c r="C22" s="11"/>
-      <c r="G22" s="12" t="str">
+      <c r="B22" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="C22" s="12"/>
+      <c r="G22" s="13" t="str">
         <f aca="false">IF(C22="","Velg i nedtrekksmenyen.",IF(C22="Lov, etikk og miljø","Riktig. En påstand som ikke er dekket av tiltak, bryter med allment aksepterte etiske normer (1.2.5).","Ikke riktig. En påstand som ikke er dekket av tiltak, bryter med allment aksepterte etiske normer (1.2.5)."))</f>
         <v>Velg i nedtrekksmenyen.</v>
       </c>
+      <c r="Z22" s="6" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="Z23" s="0" t="s">
+        <v>83</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B24" s="9" t="s">
-        <v>86</v>
-      </c>
-      <c r="C24" s="9"/>
-      <c r="D24" s="9"/>
-      <c r="E24" s="9"/>
-      <c r="F24" s="9"/>
-      <c r="G24" s="9"/>
+      <c r="B24" s="10" t="s">
+        <v>99</v>
+      </c>
+      <c r="C24" s="10"/>
+      <c r="D24" s="10"/>
+      <c r="E24" s="10"/>
+      <c r="F24" s="10"/>
+      <c r="G24" s="10"/>
+      <c r="Z24" s="6" t="s">
+        <v>84</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B25" s="10" t="s">
-        <v>87</v>
-      </c>
-      <c r="C25" s="11"/>
-      <c r="G25" s="12" t="str">
+      <c r="B25" s="11" t="s">
+        <v>100</v>
+      </c>
+      <c r="C25" s="12"/>
+      <c r="G25" s="13" t="str">
         <f aca="false">IF(C25="","Velg i nedtrekksmenyen.",IF(C25="Kjøpers marked","Riktig. Stor konkurranse: bedriftene må være lydhøre overfor kjøpernes ønsker (1.2).","Ikke riktig. Stor konkurranse: bedriftene må være lydhøre overfor kjøpernes ønsker (1.2)."))</f>
         <v>Velg i nedtrekksmenyen.</v>
       </c>
+      <c r="Z25" s="6" t="s">
+        <v>86</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B26" s="10" t="s">
-        <v>88</v>
-      </c>
-      <c r="C26" s="11"/>
-      <c r="G26" s="12" t="str">
+      <c r="B26" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="C26" s="12"/>
+      <c r="G26" s="13" t="str">
         <f aca="false">IF(C26="","Velg i nedtrekksmenyen.",IF(C26="Selgers marked","Riktig. Liten konkurranse: bedriften tar først og fremst hensyn til egne interesser (1.2). Kunden husker det i januar.","Ikke riktig. Liten konkurranse: bedriften tar først og fremst hensyn til egne interesser (1.2). Kunden husker det i januar."))</f>
         <v>Velg i nedtrekksmenyen.</v>
       </c>
+      <c r="Z26" s="6" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B27" s="10" t="s">
-        <v>89</v>
-      </c>
-      <c r="C27" s="11"/>
-      <c r="G27" s="12" t="str">
+      <c r="B27" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="C27" s="12"/>
+      <c r="G27" s="13" t="str">
         <f aca="false">IF(C27="","Velg i nedtrekksmenyen.",IF(C27="Loven er som regel bare en minimumsløsning; over den skal bedriften også tenke på det allmenne vel","Riktig. Lovgivningen representerer som regel bare minimumsløsninger; i handlingsrommet over må aktørene også tenke på det allmenne vel, ikke bare egen nytte (1.2.5.1). Lovlig er ikke det samme som bærekraftig.","Ikke riktig. Lovgivningen representerer som regel bare minimumsløsninger; i handlingsrommet over må aktørene også tenke på det allmenne vel, ikke bare egen nytte (1.2.5.1). Lovlig er ikke det samme som bærekraftig."))</f>
         <v>Velg i nedtrekksmenyen.</v>
       </c>
+      <c r="Z27" s="6" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="Z28" s="0" t="s">
+        <v>105</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B29" s="8" t="s">
-        <v>90</v>
-      </c>
-      <c r="C29" s="8"/>
-      <c r="D29" s="8"/>
-      <c r="E29" s="8"/>
-      <c r="F29" s="8"/>
-      <c r="G29" s="8"/>
+      <c r="B29" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="C29" s="9"/>
+      <c r="D29" s="9"/>
+      <c r="E29" s="9"/>
+      <c r="F29" s="9"/>
+      <c r="G29" s="9"/>
+      <c r="Z29" s="6" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B30" s="15"/>
-      <c r="C30" s="15"/>
-      <c r="D30" s="15"/>
-      <c r="E30" s="15"/>
-      <c r="F30" s="15"/>
-      <c r="G30" s="15"/>
+      <c r="B30" s="16"/>
+      <c r="C30" s="16"/>
+      <c r="D30" s="16"/>
+      <c r="E30" s="16"/>
+      <c r="F30" s="16"/>
+      <c r="G30" s="16"/>
+      <c r="Z30" s="6" t="s">
+        <v>104</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B31" s="15"/>
-      <c r="C31" s="15"/>
-      <c r="D31" s="15"/>
-      <c r="E31" s="15"/>
-      <c r="F31" s="15"/>
-      <c r="G31" s="15"/>
+      <c r="B31" s="16"/>
+      <c r="C31" s="16"/>
+      <c r="D31" s="16"/>
+      <c r="E31" s="16"/>
+      <c r="F31" s="16"/>
+      <c r="G31" s="16"/>
+      <c r="Z31" s="6" t="s">
+        <v>105</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B32" s="15"/>
-      <c r="C32" s="15"/>
-      <c r="D32" s="15"/>
-      <c r="E32" s="15"/>
-      <c r="F32" s="15"/>
-      <c r="G32" s="15"/>
+      <c r="B32" s="16"/>
+      <c r="C32" s="16"/>
+      <c r="D32" s="16"/>
+      <c r="E32" s="16"/>
+      <c r="F32" s="16"/>
+      <c r="G32" s="16"/>
+      <c r="Z32" s="6" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B33" s="16" t="str">
+      <c r="B33" s="17" t="str">
         <f aca="false">IF(LEN(B30)&lt;40,"",IF(AND(ISNUMBER(SEARCH("4",B30)),ISNUMBER(SEARCH("styret",B30))),"Bra: du bygger på forslag 4 og spør styret. Gode spørsmål handler om fordeling av kostnad og strømregning, drift om fem år og trinnvis utbygging.",IF(OR(ISNUMBER(SEARCH("4",B30)),ISNUMBER(SEARCH("styret",B30))),"Du er på sporet. Si hvilket forslag du bygger på (det som starter hos kunden), og rett spørsmålene til styret, ikke til anlegget.","Tips: bygg på forslag 4, markedsorientering. Spør styret hvordan kostnaden og strømregningen fordeles mellom beboerne, hvem som drifter anlegget om fem år, og om det kan bygges ut trinnvis.")))</f>
         <v/>
       </c>
-      <c r="C33" s="16"/>
-      <c r="D33" s="16"/>
-      <c r="E33" s="16"/>
-      <c r="F33" s="16"/>
-      <c r="G33" s="16"/>
+      <c r="C33" s="17"/>
+      <c r="D33" s="17"/>
+      <c r="E33" s="17"/>
+      <c r="F33" s="17"/>
+      <c r="G33" s="17"/>
+      <c r="Z33" s="6" t="s">
+        <v>104</v>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B34" s="17" t="s">
-        <v>42</v>
-      </c>
-      <c r="C34" s="11"/>
+      <c r="B34" s="18" t="s">
+        <v>47</v>
+      </c>
+      <c r="C34" s="12"/>
+      <c r="Z34" s="6" t="s">
+        <v>105</v>
+      </c>
     </row>
     <row r="35" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B35" s="18" t="str">
+      <c r="B35" s="19" t="str">
         <f aca="false">IF(C34="JA","Hint: Forslag 1 leter etter flere kjøpere til samme anlegg (salg). 2 tar for gitt at det beste produktet vinner (produkt). 3 handler om billig og volum (produksjon). 4 starter hos kunden (marked). 5 krever at de ansatte kan stå for løftet (helhetlig). Kravene: nettsiden mot montørene er ekstern og intern; Kystfiber er relasjon; slagordet er etikk og miljø.","")</f>
         <v/>
       </c>
-      <c r="C35" s="18"/>
-      <c r="D35" s="18"/>
-      <c r="E35" s="18"/>
-      <c r="F35" s="18"/>
-      <c r="G35" s="18"/>
+      <c r="C35" s="19"/>
+      <c r="D35" s="19"/>
+      <c r="E35" s="19"/>
+      <c r="F35" s="19"/>
+      <c r="G35" s="19"/>
+      <c r="Z35" s="6" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="Z36" s="0" t="s">
+        <v>108</v>
+      </c>
     </row>
     <row r="37" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B37" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="C37" s="6"/>
-      <c r="D37" s="6"/>
-      <c r="E37" s="6"/>
-      <c r="F37" s="6"/>
-      <c r="G37" s="6"/>
+      <c r="B37" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="C37" s="7"/>
+      <c r="D37" s="7"/>
+      <c r="E37" s="7"/>
+      <c r="F37" s="7"/>
+      <c r="G37" s="7"/>
+      <c r="Z37" s="6" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="Z38" s="0" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="Z39" s="0" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="Z40" s="0" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="Z41" s="0" t="s">
+        <v>111</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="16">
@@ -2495,47 +2987,47 @@
   </conditionalFormatting>
   <dataValidations count="12">
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C13" type="list">
-      <formula1>"Produksjonsorientering,Produktorientering,Salgsorientering,Markedsorientering,Helhetlig markedsorientering"</formula1>
+      <formula1>$Z$1:$Z$5</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C14" type="list">
-      <formula1>"Produksjonsorientering,Produktorientering,Salgsorientering,Markedsorientering,Helhetlig markedsorientering"</formula1>
+      <formula1>$Z$6:$Z$10</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C15" type="list">
-      <formula1>"Produksjonsorientering,Produktorientering,Salgsorientering,Markedsorientering,Helhetlig markedsorientering"</formula1>
+      <formula1>$Z$11:$Z$15</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C16" type="list">
-      <formula1>"Produksjonsorientering,Produktorientering,Salgsorientering,Markedsorientering,Helhetlig markedsorientering"</formula1>
+      <formula1>$Z$16:$Z$20</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C17" type="list">
-      <formula1>"Produksjonsorientering,Produktorientering,Salgsorientering,Markedsorientering,Helhetlig markedsorientering"</formula1>
+      <formula1>$Z$21:$Z$25</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C20" type="list">
-      <formula1>"Ekstern og intern markedsføring henger sammen,Relasjonsmarkedsføring,Lov,etikk og miljø"</formula1>
+      <formula1>$Z$26:$Z$28</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C21" type="list">
-      <formula1>"Ekstern og intern markedsføring henger sammen,Relasjonsmarkedsføring,Lov,etikk og miljø"</formula1>
+      <formula1>$Z$29:$Z$31</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C22" type="list">
-      <formula1>"Ekstern og intern markedsføring henger sammen,Relasjonsmarkedsføring,Lov,etikk og miljø"</formula1>
+      <formula1>$Z$32:$Z$34</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C25" type="list">
-      <formula1>"Kjøpers marked,Selgers marked"</formula1>
+      <formula1>$Z$35:$Z$36</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C26" type="list">
-      <formula1>"Kjøpers marked,Selgers marked"</formula1>
+      <formula1>$Z$37:$Z$38</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C27" type="list">
-      <formula1>"Riktig: loven bestemmer hva som er bærekraftig,Loven er som regel bare en minimumsløsning; over den skal bedriften også tenke på det allmenne vel,Bærekraft gjelder bare store selskaper"</formula1>
+      <formula1>$Z$39:$Z$41</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C34" type="list">
@@ -2568,162 +3060,162 @@
   </cols>
   <sheetData>
     <row r="2" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="25" t="s">
-        <v>91</v>
+      <c r="B2" s="26" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B3" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="C3" s="6"/>
-      <c r="D3" s="6"/>
+      <c r="B3" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="C3" s="7"/>
+      <c r="D3" s="7"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="26" t="s">
-        <v>93</v>
-      </c>
-      <c r="C5" s="26" t="s">
-        <v>94</v>
-      </c>
-      <c r="D5" s="26" t="s">
-        <v>95</v>
+      <c r="B5" s="27" t="s">
+        <v>114</v>
+      </c>
+      <c r="C5" s="27" t="s">
+        <v>115</v>
+      </c>
+      <c r="D5" s="27" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B6" s="27" t="s">
-        <v>96</v>
-      </c>
-      <c r="C6" s="23"/>
-      <c r="D6" s="27" t="s">
-        <v>97</v>
+      <c r="B6" s="28" t="s">
+        <v>117</v>
+      </c>
+      <c r="C6" s="24"/>
+      <c r="D6" s="28" t="s">
+        <v>118</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B7" s="27" t="s">
-        <v>98</v>
-      </c>
-      <c r="C7" s="23"/>
-      <c r="D7" s="27" t="s">
-        <v>99</v>
+      <c r="B7" s="28" t="s">
+        <v>119</v>
+      </c>
+      <c r="C7" s="24"/>
+      <c r="D7" s="28" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B8" s="27" t="s">
-        <v>100</v>
-      </c>
-      <c r="C8" s="23" t="n">
+      <c r="B8" s="28" t="s">
+        <v>121</v>
+      </c>
+      <c r="C8" s="24" t="n">
         <v>736</v>
       </c>
-      <c r="D8" s="27" t="s">
-        <v>101</v>
+      <c r="D8" s="28" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B9" s="27" t="s">
-        <v>102</v>
-      </c>
-      <c r="C9" s="23" t="n">
+      <c r="B9" s="28" t="s">
+        <v>123</v>
+      </c>
+      <c r="C9" s="24" t="n">
         <v>10304000</v>
       </c>
-      <c r="D9" s="27" t="s">
-        <v>103</v>
+      <c r="D9" s="28" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B10" s="27" t="s">
-        <v>104</v>
-      </c>
-      <c r="C10" s="23"/>
-      <c r="D10" s="27" t="s">
-        <v>105</v>
+      <c r="B10" s="28" t="s">
+        <v>125</v>
+      </c>
+      <c r="C10" s="24"/>
+      <c r="D10" s="28" t="s">
+        <v>126</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B11" s="27" t="s">
-        <v>106</v>
-      </c>
-      <c r="C11" s="23"/>
-      <c r="D11" s="27" t="s">
-        <v>107</v>
+      <c r="B11" s="28" t="s">
+        <v>127</v>
+      </c>
+      <c r="C11" s="24"/>
+      <c r="D11" s="28" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B12" s="27" t="s">
-        <v>108</v>
-      </c>
-      <c r="C12" s="23" t="n">
+      <c r="B12" s="28" t="s">
+        <v>129</v>
+      </c>
+      <c r="C12" s="24" t="n">
         <v>16550000</v>
       </c>
-      <c r="D12" s="27" t="s">
-        <v>109</v>
+      <c r="D12" s="28" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B13" s="27" t="s">
-        <v>110</v>
-      </c>
-      <c r="C13" s="23" t="n">
+      <c r="B13" s="28" t="s">
+        <v>131</v>
+      </c>
+      <c r="C13" s="24" t="n">
         <v>74</v>
       </c>
-      <c r="D13" s="27" t="s">
-        <v>111</v>
+      <c r="D13" s="28" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B14" s="27" t="s">
-        <v>112</v>
-      </c>
-      <c r="C14" s="23" t="n">
+      <c r="B14" s="28" t="s">
+        <v>133</v>
+      </c>
+      <c r="C14" s="24" t="n">
         <v>47</v>
       </c>
-      <c r="D14" s="27" t="s">
-        <v>113</v>
+      <c r="D14" s="28" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B15" s="27" t="s">
-        <v>114</v>
-      </c>
-      <c r="C15" s="23"/>
-      <c r="D15" s="27" t="s">
-        <v>115</v>
+      <c r="B15" s="28" t="s">
+        <v>135</v>
+      </c>
+      <c r="C15" s="24"/>
+      <c r="D15" s="28" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B16" s="27" t="s">
-        <v>116</v>
-      </c>
-      <c r="C16" s="23"/>
-      <c r="D16" s="27" t="s">
-        <v>117</v>
+      <c r="B16" s="28" t="s">
+        <v>137</v>
+      </c>
+      <c r="C16" s="24"/>
+      <c r="D16" s="28" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B17" s="27" t="s">
-        <v>118</v>
-      </c>
-      <c r="C17" s="23"/>
-      <c r="D17" s="27" t="s">
-        <v>119</v>
+      <c r="B17" s="28" t="s">
+        <v>139</v>
+      </c>
+      <c r="C17" s="24"/>
+      <c r="D17" s="28" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B18" s="27" t="s">
-        <v>120</v>
-      </c>
-      <c r="C18" s="23"/>
-      <c r="D18" s="27" t="s">
-        <v>121</v>
+      <c r="B18" s="28" t="s">
+        <v>141</v>
+      </c>
+      <c r="C18" s="24"/>
+      <c r="D18" s="28" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B19" s="27" t="s">
-        <v>122</v>
-      </c>
-      <c r="C19" s="23"/>
-      <c r="D19" s="27" t="s">
-        <v>123</v>
+      <c r="B19" s="28" t="s">
+        <v>143</v>
+      </c>
+      <c r="C19" s="24"/>
+      <c r="D19" s="28" t="s">
+        <v>144</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
LØM-appen 2.12.0: v6.1 presentasjoner per økt, realisme- og elsikkerhetsretting
</commit_message>
<xml_diff>
--- a/pensum/ma01/MA01_Hva_er_markedsforing_Oppgaver_v6.xlsx
+++ b/pensum/ma01/MA01_Hva_er_markedsforing_Oppgaver_v6.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="147">
   <si>
     <t xml:space="preserve">Hva er markedsføring? Oppgaver til kapittel 1</t>
   </si>
@@ -74,7 +74,7 @@
     <t xml:space="preserve">Mellomhandlermarkedet</t>
   </si>
   <si>
-    <t xml:space="preserve">Alene, i par eller i gruppe, slik du vil.</t>
+    <t xml:space="preserve">Del 1, de åtte forespørslene, hører til økt 2 av 3 (hovedmarkedene). Del 2, fra «Marked betyr tre ting», hører til økt 1 av 3 (markedsføring og marked). Alene, i par eller i gruppe, slik du vil.</t>
   </si>
   <si>
     <t xml:space="preserve">Det offentlige markedet</t>
@@ -110,7 +110,7 @@
     <t xml:space="preserve">1 Huseier: ladepunkt i egen garasje, til eget bruk</t>
   </si>
   <si>
-    <t xml:space="preserve">2 Kystfiber Entreprenør AS: elektro i et næringsbygg de bygger for en kunde</t>
+    <t xml:space="preserve">2 Haugerud Bygg AS: elektro i et næringsbygg de bygger for en kunde</t>
   </si>
   <si>
     <t xml:space="preserve">3 Kommunen: elektro på ny skole, lyst ut som anbud</t>
@@ -122,13 +122,13 @@
     <t xml:space="preserve">5 Byggvarehus: kjøper montering av ladepunkt og selger den videre i pakke</t>
   </si>
   <si>
-    <t xml:space="preserve">6 Fjellkraft Nett AS, aksjeselskap eid av kommunen: målerbytte etter rammeavtale</t>
+    <t xml:space="preserve">6 Fjellkraft Nett AS, aksjeselskap eid av kommunen: lavspenningsarbeid etter rammeavtale</t>
   </si>
   <si>
     <t xml:space="preserve">7 Kruttverket Utvikling AS, byggherre: elektro i nytt kontorbygg med lager</t>
   </si>
   <si>
-    <t xml:space="preserve">8 Statens vegvesen: nytt lys i en tunnel</t>
+    <t xml:space="preserve">8 Fylkeskommunen: ny belysning og nødlys i en videregående skole, kunngjort i Doffin</t>
   </si>
   <si>
     <t xml:space="preserve">Marked betyr tre ting</t>
@@ -185,6 +185,9 @@
     <t xml:space="preserve">Oppgave 1B: Nordlys' markeder: hvor avhengig er Kari av byggherrene?</t>
   </si>
   <si>
+    <t xml:space="preserve">Økt 2 av 3, de fem hovedmarkedene. Alene, i par eller i gruppe, slik du vil.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Kari skal lage budsjett for 2027 og vil vite hvor pengene kommer fra. Ida har satt opp salgsinntekten for 2026, 22 400 000 kr, på seks kundegrupper. Plasser gruppene i hovedmarked, regn bedriftsmarkedet og byggherrenes andel, og sammenlikn med bransjen, der 59,6 % av omsetningen kom fra næringsbygg og nye boliger og 19,7 % fra service i 2025 (NHO Elektro, bransjeforeningen for elektrobedriftene i Næringslivets Hovedorganisasjon, lønnsomhetsrapport 2025).</t>
   </si>
   <si>
@@ -209,7 +212,7 @@
     <t xml:space="preserve">Næringskunder, service og prosjekt (butikker, verksteder, kontorer)</t>
   </si>
   <si>
-    <t xml:space="preserve">Fjellkraft Nett AS, rammeavtale om målerbytte</t>
+    <t xml:space="preserve">Fjellkraft Nett AS, rammeavtale om lavspenningsarbeid</t>
   </si>
   <si>
     <t xml:space="preserve">Kommunen og fylkeskommunen, anbud (skoler, barnehager)</t>
@@ -278,13 +281,16 @@
     <t xml:space="preserve">Produktorientering</t>
   </si>
   <si>
+    <t xml:space="preserve">Økt 3 av 3, grunnholdningene. Alene, i par eller i gruppe, slik du vil.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Salgsorientering</t>
   </si>
   <si>
     <t xml:space="preserve">Markedsorientering</t>
   </si>
   <si>
-    <t xml:space="preserve">I fjor leverte Ida tre anbud på ladeanlegg til borettslag og vant ingen av dem, selv om Nordlys' anlegg ble vurdert som teknisk best alle tre gangene. Det er 22 borettslag i nedslagsfeltet. På mandagsmøtet kommer fem forslag til hva Nordlys skal gjøre. Samtidig har Kari skrevet et løfte på nettsiden, Kystfiber vil samarbeide, og Fjell Elektro vurderer et slagord. Sett navn på grunnholdningene og kravene, og skriv spørsmålene Ida bør stille styret.</t>
+    <t xml:space="preserve">I fjor leverte Ida tre anbud på ladeanlegg til borettslag og vant ingen av dem, selv om styret sa at anlegget var godt alle tre gangene. Det er 22 borettslag i nedslagsfeltet. På mandagsmøtet kommer fem forslag til hva Nordlys skal gjøre. Samtidig har Kari skrevet et løfte på nettsiden, Kystfiber vil samarbeide, og Fjell Elektro vurderer et slagord. Sett navn på grunnholdningene og kravene, og skriv spørsmålene Ida bør stille styret.</t>
   </si>
   <si>
     <t xml:space="preserve">Helhetlig markedsorientering</t>
@@ -329,10 +335,10 @@
     <t xml:space="preserve">Kjøpers eller selgers marked, og bærekraft (velg i nedtrekksmenyen)</t>
   </si>
   <si>
-    <t xml:space="preserve">Januar hos Nordlys: tynn ordrebok, mange ledige montører i byen, kunden forhandler ned prisen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mai hos Nordlys: alle vil ha ladepunkt før ferien, og Nordlys setter leveringstiden</t>
+    <t xml:space="preserve">August hos Nordlys: tynn ordrebok, mange ledige montører i byen, kunden forhandler ned prisen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oktober hos Nordlys: alle vil ha ladepunkt før jul, og Nordlys setter leveringstiden</t>
   </si>
   <si>
     <t xml:space="preserve">Ekstern og intern markedsføring henger sammen</t>
@@ -383,7 +389,7 @@
     <t xml:space="preserve">1A Hovedmarkedene</t>
   </si>
   <si>
-    <t xml:space="preserve">Forbrukermarkedet: 1 huseier. Bedriftsmarkedet: 2 Kystfiber, 6 Fjellkraft Nett (offentlig næringsdrift), 7 Kruttverket Utvikling. Det offentlige markedet: 3 kommunen, 8 Statens vegvesen. Organisasjonsmarkedet: 4 idrettslaget. Mellomhandlermarkedet: 5 byggvarehuset.</t>
+    <t xml:space="preserve">Forbrukermarkedet: 1 huseier. Bedriftsmarkedet: 2 Haugerud, 6 Fjellkraft Nett (offentlig næringsdrift), 7 Kruttverket Utvikling. Det offentlige markedet: 3 kommunen, 8 fylkeskommunen. Organisasjonsmarkedet: 4 idrettslaget. Mellomhandlermarkedet: 5 byggvarehuset.</t>
   </si>
   <si>
     <t xml:space="preserve">1A Betydningene</t>
@@ -437,7 +443,7 @@
     <t xml:space="preserve">1B d) Svaret til Kari</t>
   </si>
   <si>
-    <t xml:space="preserve">Nesten halve omsetningen, 47 %, kommer fra byggherrer og entreprenører, én kundegruppe som stopper når boligbyggingen stopper. Bransjen henter 59,6 % der. Vekst kan ligge i service hos husstander og næringskunder (bransjen: 19,7 %) eller i anbud i det offentlige markedet; de kjøper annerledes enn byggherrene og må få et annet tilbud.</t>
+    <t xml:space="preserve">Nesten halve omsetningen, 47 %, kommer fra byggherrer og entreprenører, én kundegruppe som stopper når byggeaktiviteten faller. Bransjen henter 59,6 % fra hele nybyggmarkedet; med kommunens nybygg er Nordlys oppe i 64 %. Vekst kan ligge i service hos husstander og næringskunder (bransjen: 19,7 %) eller i rammeavtaler om drift og vedlikehold i det offentlige markedet; de kjøper annerledes enn byggherrene og må få et annet tilbud.</t>
   </si>
   <si>
     <t xml:space="preserve">1C Forslagene</t>
@@ -455,7 +461,7 @@
     <t xml:space="preserve">1C Marked og bærekraft</t>
   </si>
   <si>
-    <t xml:space="preserve">Januar: kjøpers marked. Mai: selgers marked. Loven er som regel bare en minimumsløsning; over den skal bedriften også tenke på det allmenne vel.</t>
+    <t xml:space="preserve">August: kjøpers marked. Oktober: selgers marked. Loven er som regel bare en minimumsløsning; over den skal bedriften også tenke på det allmenne vel.</t>
   </si>
   <si>
     <t xml:space="preserve">1C Spørsmålene til styret</t>
@@ -1150,7 +1156,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="7" t="s">
         <v>16</v>
       </c>
@@ -1361,7 +1367,7 @@
       </c>
       <c r="C20" s="12"/>
       <c r="G20" s="13" t="str">
-        <f aca="false">IF(C20="","Velg i nedtrekksmenyen.",IF(C20="Det offentlige markedet","Riktig. Statlig forvaltning: departementer, direktorater og etater (1.4.3).","Ikke riktig. Statlig forvaltning: departementer, direktorater og etater (1.4.3)."))</f>
+        <f aca="false">IF(C20="","Velg i nedtrekksmenyen.",IF(C20="Det offentlige markedet","Riktig. Offentlig forvaltning som kjøper etter anskaffelsesregelverket, med kunngjøring i Doffin (1.4.3).","Ikke riktig. Offentlig forvaltning som kjøper etter anskaffelsesregelverket, med kunngjøring i Doffin (1.4.3)."))</f>
         <v>Velg i nedtrekksmenyen.</v>
       </c>
       <c r="Z20" s="6" t="s">
@@ -1868,7 +1874,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="7" t="s">
-        <v>16</v>
+        <v>53</v>
       </c>
       <c r="C3" s="7"/>
       <c r="D3" s="7"/>
@@ -1894,7 +1900,7 @@
     </row>
     <row r="5" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="9" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C5" s="9"/>
       <c r="D5" s="9"/>
@@ -1920,7 +1926,7 @@
     </row>
     <row r="7" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="9" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C7" s="9"/>
       <c r="D7" s="9"/>
@@ -1938,7 +1944,7 @@
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B9" s="8" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C9" s="8"/>
       <c r="D9" s="8"/>
@@ -1951,7 +1957,7 @@
     </row>
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="9" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C10" s="9"/>
       <c r="D10" s="9"/>
@@ -1964,10 +1970,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="20" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C11" s="21" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="Z11" s="6" t="s">
         <v>13</v>
@@ -1975,7 +1981,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="22" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C12" s="23" t="n">
         <v>10500000</v>
@@ -1986,7 +1992,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="22" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C13" s="23" t="n">
         <v>4400000</v>
@@ -1997,7 +2003,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="22" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C14" s="23" t="n">
         <v>1650000</v>
@@ -2008,7 +2014,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="22" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C15" s="23" t="n">
         <v>3800000</v>
@@ -2019,7 +2025,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="22" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C16" s="23" t="n">
         <v>1450000</v>
@@ -2030,7 +2036,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="22" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C17" s="23" t="n">
         <v>600000</v>
@@ -2041,7 +2047,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="22" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C18" s="24" t="n">
         <f aca="false">SUM(C12:C17)</f>
@@ -2058,7 +2064,7 @@
     </row>
     <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B20" s="8" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C20" s="8"/>
       <c r="D20" s="8"/>
@@ -2071,7 +2077,7 @@
     </row>
     <row r="21" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B21" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C21" s="9"/>
       <c r="D21" s="9"/>
@@ -2089,7 +2095,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B23" s="10" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C23" s="10"/>
       <c r="D23" s="10"/>
@@ -2102,7 +2108,7 @@
     </row>
     <row r="24" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B24" s="11" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C24" s="12"/>
       <c r="G24" s="13" t="str">
@@ -2115,7 +2121,7 @@
     </row>
     <row r="25" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B25" s="11" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C25" s="12"/>
       <c r="G25" s="13" t="str">
@@ -2128,7 +2134,7 @@
     </row>
     <row r="26" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B26" s="11" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C26" s="12"/>
       <c r="G26" s="13" t="str">
@@ -2141,7 +2147,7 @@
     </row>
     <row r="27" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B27" s="11" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C27" s="12"/>
       <c r="G27" s="13" t="str">
@@ -2154,7 +2160,7 @@
     </row>
     <row r="28" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B28" s="11" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C28" s="12"/>
       <c r="G28" s="13" t="str">
@@ -2167,7 +2173,7 @@
     </row>
     <row r="29" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B29" s="11" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C29" s="12"/>
       <c r="G29" s="13" t="str">
@@ -2185,7 +2191,7 @@
     </row>
     <row r="31" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B31" s="11" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C31" s="14"/>
       <c r="D31" s="15" t="s">
@@ -2198,11 +2204,11 @@
     </row>
     <row r="32" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B32" s="11" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C32" s="25"/>
       <c r="D32" s="15" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="G32" s="13" t="str">
         <f aca="false">IF(C32="","Skriv svaret i den gule cellen.",IF(C32=(ROUND((C12+C13+C14)/C18*100,0)),"Riktig.",IF(ABS(C32-(ROUND(C12/C18*100,0)))&lt;=0,"Det er byggherrenes andel alene. Her skal hele bedriftsmarkedet (a) deles på salgsinntekten.",IF(ABS(C32-(ROUND((C12+C13+C14+C15)/C18*100,0)))&lt;=0,"Du har tatt med kommunen i bedriftsmarkedet. Kommunen er det offentlige markedet.","Ikke riktig ennå. Se på regnestykket øverst på fanen, og sjekk at du har med alle leddene."))))</f>
@@ -2211,11 +2217,11 @@
     </row>
     <row r="33" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B33" s="11" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C33" s="25"/>
       <c r="D33" s="15" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="G33" s="13" t="str">
         <f aca="false">IF(C33="","Skriv svaret i den gule cellen.",IF(C33=(ROUND(C12/C18*100,0)),"Riktig.",IF(ABS(C33-(ROUND(C12/(C12+C13+C14)*100,0)))&lt;=0,"Du har delt på bedriftsmarkedet, 16 550 000. Andelen skal regnes av hele salgsinntekten, 22 400 000.",IF(ABS(C33-(60))&lt;=0,"Det er bransjens tall, 59,6 %. Her spør vi om Nordlys: 10 500 000 delt på 22 400 000.","Ikke riktig ennå. Se på regnestykket øverst på fanen, og sjekk at du har med alle leddene."))))</f>
@@ -2224,7 +2230,7 @@
     </row>
     <row r="35" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B35" s="9" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C35" s="9"/>
       <c r="D35" s="9"/>
@@ -2258,7 +2264,7 @@
     </row>
     <row r="39" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B39" s="17" t="str">
-        <f aca="false">IF(LEN(B36)&lt;40,"",IF(AND(ISNUMBER(SEARCH("byggherre",B36)),ISNUMBER(SEARCH("47",B36))),"Bra: du bruker 47 % og peker på byggherrene. Sjekk at du også sier hvilket marked du ville vokse i, og hvorfor det kjøper annerledes.",IF(OR(ISNUMBER(SEARCH("byggherre",B36)),ISNUMBER(SEARCH("47",B36))),"Du er på sporet. Bruk tallet: byggherrene er 47 % av salgsinntekten, mot 59,6 % i bransjen. Si hva som skjer når boligbyggingen stopper, og hvor du ville vokse.","Tips: 47 % av salgsinntekten kommer fra byggherrer og entreprenører, én kundegruppe som stopper når boligbyggingen stopper. Bransjen henter 59,6 % der, så Nordlys er litt mindre utsatt, men nesten halve omsetningen er i spill. Vekst kan ligge i service hos husstander og næringskunder, eller i anbud i det offentlige markedet.")))</f>
+        <f aca="false">IF(LEN(B36)&lt;40,"",IF(AND(ISNUMBER(SEARCH("byggherre",B36)),ISNUMBER(SEARCH("47",B36))),"Bra: du bruker 47 % og peker på byggherrene. Sjekk at du også sier hvilket marked du ville vokse i, og hvorfor det kjøper annerledes.",IF(OR(ISNUMBER(SEARCH("byggherre",B36)),ISNUMBER(SEARCH("47",B36))),"Du er på sporet. Bruk tallet: byggherrene er 47 % av salgsinntekten, mot 59,6 % i bransjen. Si hva som skjer når byggeaktiviteten faller, og hvor du ville vokse.","Tips: 47 % av salgsinntekten kommer fra byggherrer og entreprenører, én kundegruppe som stopper når byggeaktiviteten faller. Bransjen henter 59,6 % fra næringsbygg og nye boliger, men det tallet omfatter hele nybyggmarkedet; med kommunens skoler og barnehager er Nordlys oppe i 64 %, så nesten to tredeler er i spill når byggeaktiviteten faller. Vekst kan ligge i service hos husstander og næringskunder, eller i rammeavtaler om drift og vedlikehold i det offentlige markedet.")))</f>
         <v/>
       </c>
       <c r="C39" s="17"/>
@@ -2443,12 +2449,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="Z1" s="0" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="5" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C2" s="5"/>
       <c r="D2" s="5"/>
@@ -2456,12 +2462,12 @@
       <c r="F2" s="5"/>
       <c r="G2" s="5"/>
       <c r="Z2" s="6" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="7" t="s">
-        <v>16</v>
+        <v>84</v>
       </c>
       <c r="C3" s="7"/>
       <c r="D3" s="7"/>
@@ -2469,7 +2475,7 @@
       <c r="F3" s="7"/>
       <c r="G3" s="7"/>
       <c r="Z3" s="6" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2482,12 +2488,12 @@
       <c r="F4" s="8"/>
       <c r="G4" s="8"/>
       <c r="Z4" s="6" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="9" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C5" s="9"/>
       <c r="D5" s="9"/>
@@ -2495,7 +2501,7 @@
       <c r="F5" s="9"/>
       <c r="G5" s="9"/>
       <c r="Z5" s="6" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2508,12 +2514,12 @@
       <c r="F6" s="8"/>
       <c r="G6" s="8"/>
       <c r="Z6" s="6" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="9" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C7" s="9"/>
       <c r="D7" s="9"/>
@@ -2521,12 +2527,12 @@
       <c r="F7" s="9"/>
       <c r="G7" s="9"/>
       <c r="Z7" s="6" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="Z8" s="0" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2539,12 +2545,12 @@
       <c r="F9" s="8"/>
       <c r="G9" s="8"/>
       <c r="Z9" s="6" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="9" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C10" s="9"/>
       <c r="D10" s="9"/>
@@ -2552,17 +2558,17 @@
       <c r="F10" s="9"/>
       <c r="G10" s="9"/>
       <c r="Z10" s="6" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="Z11" s="0" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="10" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C12" s="10"/>
       <c r="D12" s="10"/>
@@ -2570,12 +2576,12 @@
       <c r="F12" s="10"/>
       <c r="G12" s="10"/>
       <c r="Z12" s="6" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="11" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C13" s="12"/>
       <c r="G13" s="13" t="str">
@@ -2583,12 +2589,12 @@
         <v>Velg i nedtrekksmenyen.</v>
       </c>
       <c r="Z13" s="6" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B14" s="11" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C14" s="12"/>
       <c r="G14" s="13" t="str">
@@ -2596,12 +2602,12 @@
         <v>Velg i nedtrekksmenyen.</v>
       </c>
       <c r="Z14" s="6" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B15" s="11" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C15" s="12"/>
       <c r="G15" s="13" t="str">
@@ -2609,12 +2615,12 @@
         <v>Velg i nedtrekksmenyen.</v>
       </c>
       <c r="Z15" s="6" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="11" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C16" s="12"/>
       <c r="G16" s="13" t="str">
@@ -2622,12 +2628,12 @@
         <v>Velg i nedtrekksmenyen.</v>
       </c>
       <c r="Z16" s="6" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B17" s="11" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C17" s="12"/>
       <c r="G17" s="13" t="str">
@@ -2635,17 +2641,17 @@
         <v>Velg i nedtrekksmenyen.</v>
       </c>
       <c r="Z17" s="6" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="Z18" s="0" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B19" s="10" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C19" s="10"/>
       <c r="D19" s="10"/>
@@ -2653,12 +2659,12 @@
       <c r="F19" s="10"/>
       <c r="G19" s="10"/>
       <c r="Z19" s="6" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B20" s="11" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C20" s="12"/>
       <c r="G20" s="13" t="str">
@@ -2666,12 +2672,12 @@
         <v>Velg i nedtrekksmenyen.</v>
       </c>
       <c r="Z20" s="6" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B21" s="11" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C21" s="12"/>
       <c r="G21" s="13" t="str">
@@ -2679,12 +2685,12 @@
         <v>Velg i nedtrekksmenyen.</v>
       </c>
       <c r="Z21" s="6" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B22" s="11" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C22" s="12"/>
       <c r="G22" s="13" t="str">
@@ -2692,17 +2698,17 @@
         <v>Velg i nedtrekksmenyen.</v>
       </c>
       <c r="Z22" s="6" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="Z23" s="0" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B24" s="10" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C24" s="10"/>
       <c r="D24" s="10"/>
@@ -2710,12 +2716,12 @@
       <c r="F24" s="10"/>
       <c r="G24" s="10"/>
       <c r="Z24" s="6" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B25" s="11" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C25" s="12"/>
       <c r="G25" s="13" t="str">
@@ -2723,25 +2729,25 @@
         <v>Velg i nedtrekksmenyen.</v>
       </c>
       <c r="Z25" s="6" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B26" s="11" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C26" s="12"/>
       <c r="G26" s="13" t="str">
-        <f aca="false">IF(C26="","Velg i nedtrekksmenyen.",IF(C26="Selgers marked","Riktig. Liten konkurranse: bedriften tar først og fremst hensyn til egne interesser (1.2). Kunden husker det i januar.","Ikke riktig. Liten konkurranse: bedriften tar først og fremst hensyn til egne interesser (1.2). Kunden husker det i januar."))</f>
+        <f aca="false">IF(C26="","Velg i nedtrekksmenyen.",IF(C26="Selgers marked","Riktig. Liten konkurranse: bedriften tar først og fremst hensyn til egne interesser (1.2). Kunden husker det i august.","Ikke riktig. Liten konkurranse: bedriften tar først og fremst hensyn til egne interesser (1.2). Kunden husker det i august."))</f>
         <v>Velg i nedtrekksmenyen.</v>
       </c>
       <c r="Z26" s="6" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B27" s="11" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C27" s="12"/>
       <c r="G27" s="13" t="str">
@@ -2749,17 +2755,17 @@
         <v>Velg i nedtrekksmenyen.</v>
       </c>
       <c r="Z27" s="6" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="Z28" s="0" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B29" s="9" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C29" s="9"/>
       <c r="D29" s="9"/>
@@ -2767,7 +2773,7 @@
       <c r="F29" s="9"/>
       <c r="G29" s="9"/>
       <c r="Z29" s="6" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2778,7 +2784,7 @@
       <c r="F30" s="16"/>
       <c r="G30" s="16"/>
       <c r="Z30" s="6" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2789,7 +2795,7 @@
       <c r="F31" s="16"/>
       <c r="G31" s="16"/>
       <c r="Z31" s="6" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2800,7 +2806,7 @@
       <c r="F32" s="16"/>
       <c r="G32" s="16"/>
       <c r="Z32" s="6" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2814,7 +2820,7 @@
       <c r="F33" s="17"/>
       <c r="G33" s="17"/>
       <c r="Z33" s="6" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2823,7 +2829,7 @@
       </c>
       <c r="C34" s="12"/>
       <c r="Z34" s="6" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2837,12 +2843,12 @@
       <c r="F35" s="19"/>
       <c r="G35" s="19"/>
       <c r="Z35" s="6" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="Z36" s="0" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2855,27 +2861,27 @@
       <c r="F37" s="7"/>
       <c r="G37" s="7"/>
       <c r="Z37" s="6" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="Z38" s="0" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="Z39" s="0" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="Z40" s="0" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="Z41" s="0" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
   </sheetData>
@@ -3061,161 +3067,161 @@
   <sheetData>
     <row r="2" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="26" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="7" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C3" s="7"/>
       <c r="D3" s="7"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="27" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C5" s="27" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="D5" s="27" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="28" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C6" s="24"/>
       <c r="D6" s="28" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="28" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C7" s="24"/>
       <c r="D7" s="28" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="28" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C8" s="24" t="n">
         <v>736</v>
       </c>
       <c r="D8" s="28" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B9" s="28" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="C9" s="24" t="n">
         <v>10304000</v>
       </c>
       <c r="D9" s="28" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="28" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C10" s="24"/>
       <c r="D10" s="28" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B11" s="28" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C11" s="24"/>
       <c r="D11" s="28" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="28" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C12" s="24" t="n">
         <v>16550000</v>
       </c>
       <c r="D12" s="28" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="28" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C13" s="24" t="n">
         <v>74</v>
       </c>
       <c r="D13" s="28" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B14" s="28" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="C14" s="24" t="n">
         <v>47</v>
       </c>
       <c r="D14" s="28" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B15" s="28" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C15" s="24"/>
       <c r="D15" s="28" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="28" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C16" s="24"/>
       <c r="D16" s="28" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B17" s="28" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C17" s="24"/>
       <c r="D17" s="28" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B18" s="28" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="C18" s="24"/>
       <c r="D18" s="28" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B19" s="28" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C19" s="24"/>
       <c r="D19" s="28" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Regneark: radhøyder og tekstbryting rettet i 53 xlsx (radhoyde.py)
</commit_message>
<xml_diff>
--- a/pensum/ma01/MA01_Hva_er_markedsforing_Oppgaver_v6.xlsx
+++ b/pensum/ma01/MA01_Hva_er_markedsforing_Oppgaver_v6.xlsx
@@ -654,7 +654,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -769,6 +769,10 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment wrapText="true" horizontal="general" vertical="bottom" textRotation="0" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -1056,7 +1060,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row ht="17.25" customHeight="true" r="5" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="3" t="s">
         <v>2</v>
       </c>
@@ -1081,27 +1085,27 @@
         <v>6</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row ht="17.25" customHeight="true" r="11" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row ht="17.25" customHeight="true" r="12" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row ht="17.25" customHeight="true" r="13" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row ht="17.25" customHeight="true" r="14" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row ht="17.25" customHeight="true" r="15" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="2" t="s">
         <v>11</v>
       </c>
@@ -1257,7 +1261,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row ht="17.25" customHeight="true" r="12" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="10" t="s">
         <v>26</v>
       </c>
@@ -1990,8 +1994,8 @@
         <v>15</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="22" t="s">
+    <row ht="31.5" customHeight="true" r="13" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+      <c s="29" r="B13" t="s">
         <v>61</v>
       </c>
       <c r="C13" s="23" t="n">
@@ -2001,8 +2005,8 @@
         <v>17</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="22" t="s">
+    <row ht="31.5" customHeight="true" r="14" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+      <c s="29" r="B14" t="s">
         <v>62</v>
       </c>
       <c r="C14" s="23" t="n">
@@ -2012,8 +2016,8 @@
         <v>19</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="22" t="s">
+    <row ht="31.5" customHeight="true" r="15" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+      <c s="29" r="B15" t="s">
         <v>63</v>
       </c>
       <c r="C15" s="23" t="n">
@@ -2023,8 +2027,8 @@
         <v>21</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="22" t="s">
+    <row ht="31.5" customHeight="true" r="16" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+      <c s="29" r="B16" t="s">
         <v>64</v>
       </c>
       <c r="C16" s="23" t="n">
@@ -2075,7 +2079,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row ht="75.75" customHeight="true" r="21" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="9" t="s">
         <v>68</v>
       </c>
@@ -2093,7 +2097,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row ht="17.25" customHeight="true" r="23" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="10" t="s">
         <v>69</v>
       </c>
@@ -2566,7 +2570,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row ht="17.25" customHeight="true" r="12" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="10" t="s">
         <v>91</v>
       </c>
@@ -2649,7 +2653,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row ht="17.25" customHeight="true" r="19" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="10" t="s">
         <v>97</v>
       </c>
@@ -2662,7 +2666,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row ht="46.5" customHeight="true" r="20" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="11" t="s">
         <v>98</v>
       </c>
@@ -2688,7 +2692,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row ht="46.5" customHeight="true" r="22" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="11" t="s">
         <v>100</v>
       </c>
@@ -2706,7 +2710,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row ht="17.25" customHeight="true" r="24" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="10" t="s">
         <v>101</v>
       </c>

</xml_diff>